<commit_message>
v0.00.001 feat(SHBS-25): Taster S2 auf liegenden C&K PTS645VL58-2 LFS umgestellt
Neuer Bauteilordner pcb/Bauteile/PTS645VL58-2LFS mit KiCad-Footprint und
Herstellermodell (kicad-packages3D), in fp-lib-table eingetragen. S2 im
Schaltplan: Footprint, Wert, Hersteller, Bestellnummern (Mouser
611-PTS645VL582, DigiKey CKN9116-ND); Altfelder des Bourns-Imports
bereinigt. Stücklisten-Generator kennt den neuen THT-Footprint,
Stückliste neu erzeugt. ERC unverändert.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/pcb/BasisStation_Stueckliste.xlsx
+++ b/pcb/BasisStation_Stueckliste.xlsx
@@ -538,7 +538,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Quelle: pcb/BasisStation/*.kicad_sch · Stand 2026-09-24 · 44 Positionen · 78 Bauteile</t>
+          <t>Quelle: pcb/BasisStation/*.kicad_sch · Stand 2026-09-29 · 44 Positionen · 78 Bauteile</t>
         </is>
       </c>
     </row>
@@ -4442,7 +4442,7 @@
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>1543-650-149</t>
+          <t>PTS645VL58-2 LFS</t>
         </is>
       </c>
       <c r="E44" s="4" t="inlineStr">
@@ -4452,34 +4452,46 @@
       </c>
       <c r="F44" s="4" t="inlineStr">
         <is>
-          <t>1543-650-149:1543650149</t>
+          <t>PTS645VL58-2LFS:SW_Tactile_SPST_Angled_PTS645Vx58-2LFS</t>
         </is>
       </c>
       <c r="G44" s="4" t="inlineStr">
         <is>
-          <t>Bourns</t>
+          <t>C&amp;K</t>
         </is>
       </c>
       <c r="H44" s="4" t="inlineStr">
         <is>
-          <t>1543-650-149</t>
+          <t>PTS645VL58-2 LFS</t>
         </is>
       </c>
       <c r="I44" s="4" t="inlineStr">
         <is>
-          <t>652-1543-650-149</t>
-        </is>
-      </c>
-      <c r="J44" s="6" t="n">
-        <v>1.17</v>
+          <t>611-PTS645VL582</t>
+        </is>
+      </c>
+      <c r="J44" s="7" t="n">
+        <v>0.284</v>
       </c>
       <c r="K44" s="4" t="n">
-        <v>412</v>
-      </c>
-      <c r="L44" s="4" t="n"/>
-      <c r="M44" s="8" t="n"/>
-      <c r="N44" s="4" t="n"/>
-      <c r="O44" s="4" t="inlineStr"/>
+        <v>290</v>
+      </c>
+      <c r="L44" s="4" t="inlineStr">
+        <is>
+          <t>CKN9116-ND</t>
+        </is>
+      </c>
+      <c r="M44" s="6" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="N44" s="4" t="n">
+        <v>19085</v>
+      </c>
+      <c r="O44" s="4" t="inlineStr">
+        <is>
+          <t>Aktiv</t>
+        </is>
+      </c>
       <c r="P44" s="4" t="inlineStr">
         <is>
           <t>Mouser</t>
@@ -4498,7 +4510,11 @@
           <t>Mouser</t>
         </is>
       </c>
-      <c r="T44" s="4" t="n"/>
+      <c r="T44" s="9" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
       <c r="U44" s="9" t="inlineStr">
         <is>
           <t>PDF</t>
@@ -4509,11 +4525,7 @@
           <t>eindeutig</t>
         </is>
       </c>
-      <c r="W44" s="5" t="inlineStr">
-        <is>
-          <t>Bei DigiKey nicht geführt — nur über Mouser.</t>
-        </is>
-      </c>
+      <c r="W44" s="5" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="4" t="n">
@@ -5177,22 +5189,23 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T43" r:id="rId113"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U43" r:id="rId114"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S44" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U44" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S45" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T45" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U45" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S46" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T46" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U46" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S47" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T47" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U47" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S48" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T48" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U48" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S49" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T49" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U49" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T44" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U44" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S45" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T45" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U45" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S46" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T46" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U46" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S47" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T47" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U47" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S48" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T48" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U48" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S49" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T49" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U49" r:id="rId132"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5228,7 +5241,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Alle 78 bestückten Referenzen einzeln · Stand 2026-09-24</t>
+          <t>Alle 78 bestückten Referenzen einzeln · Stand 2026-09-29</t>
         </is>
       </c>
     </row>
@@ -6296,7 +6309,7 @@
       </c>
       <c r="B28" s="15" t="inlineStr">
         <is>
-          <t>1543-650-149</t>
+          <t>PTS645VL58-2 LFS</t>
         </is>
       </c>
       <c r="C28" s="15" t="inlineStr">
@@ -6316,22 +6329,22 @@
       </c>
       <c r="F28" s="15" t="inlineStr">
         <is>
-          <t>1543-650-149:1543650149</t>
+          <t>PTS645VL58-2LFS:SW_Tactile_SPST_Angled_PTS645Vx58-2LFS</t>
         </is>
       </c>
       <c r="G28" s="15" t="inlineStr">
         <is>
-          <t>Bourns</t>
+          <t>C&amp;K</t>
         </is>
       </c>
       <c r="H28" s="15" t="inlineStr">
         <is>
-          <t>1543-650-149</t>
+          <t>PTS645VL58-2 LFS</t>
         </is>
       </c>
       <c r="I28" s="15" t="inlineStr">
         <is>
-          <t>652-1543-650-149</t>
+          <t>611-PTS645VL582</t>
         </is>
       </c>
     </row>
@@ -8944,7 +8957,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Stand 2026-09-24 · Der Schaltplan ist elektrisch fertig (ERC 0 Fehler).</t>
+          <t>Stand 2026-09-29 · Der Schaltplan ist elektrisch fertig (ERC 0 Fehler).</t>
         </is>
       </c>
     </row>
@@ -8988,12 +9001,12 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>5 Positionen nur bei einem Anbieter</t>
+          <t>4 Positionen nur bei einem Anbieter</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>C23 (nur Mouser); C25, C26 (nur Mouser); FB1 (nur DigiKey); R19, R20, R21, R22 (nur Mouser); S2 (nur Mouser)</t>
+          <t>C23 (nur Mouser); C25, C26 (nur Mouser); FB1 (nur DigiKey); R19, R20, R21, R22 (nur Mouser)</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">

</xml_diff>

<commit_message>
v0.00.001 docs(SHBS-43): LED-Ansteuerung, Layout und Stückliste dokumentiert
hardware.md (Status-LEDs, liegende Montage, Gesamt-Layout, DRC),
power_supply.md (Platzierung Buck-Wandler, +3V3-Verteilung),
Stückliste neu erzeugt, Report zum Hardware-Review.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/pcb/BasisStation_Stueckliste.xlsx
+++ b/pcb/BasisStation_Stueckliste.xlsx
@@ -12,8 +12,8 @@
     <sheet name="Offene Punkte" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Stückliste'!$A$5:$W$49</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Einzelpositionen'!$A$5:$I$83</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Stückliste'!$A$5:$W$46</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Einzelpositionen'!$A$5:$I$75</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -500,7 +500,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W55"/>
+  <dimension ref="A1:W52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -538,7 +538,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Quelle: pcb/BasisStation/*.kicad_sch · Stand 2026-09-29 · 44 Positionen · 78 Bauteile</t>
+          <t>Quelle: pcb/BasisStation/*.kicad_sch · Stand 2026-09-30 · 41 Positionen · 70 Bauteile</t>
         </is>
       </c>
     </row>
@@ -1964,12 +1964,12 @@
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>THT</t>
+          <t>SMD</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>WL-TMRC_3MM:WL-TMRC_3MM</t>
+          <t>LED_THT:LED_D3.0mm_Horizontal_O1.27mm_Z2.0mm</t>
         </is>
       </c>
       <c r="G19" s="4" t="inlineStr">
@@ -2063,12 +2063,12 @@
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>THT</t>
+          <t>SMD</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>WL-TMRW_3MM:WL-TMRW_3MM</t>
+          <t>LED_THT:LED_D3.0mm_Horizontal_O1.27mm_Z2.0mm</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr">
@@ -2162,12 +2162,12 @@
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>THT</t>
+          <t>SMD</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>WL-TMRW_3MM:WL-TMRW_3MM</t>
+          <t>LED_THT:LED_D3.0mm_Horizontal_O1.27mm_Z2.0mm</t>
         </is>
       </c>
       <c r="G21" s="4" t="inlineStr">
@@ -2261,12 +2261,12 @@
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>THT</t>
+          <t>SMD</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>WL-TMRC_3MM:WL-TMRC_3MM</t>
+          <t>LED_THT:LED_D3.0mm_Horizontal_O1.27mm_Z2.0mm</t>
         </is>
       </c>
       <c r="G22" s="4" t="inlineStr">
@@ -3142,59 +3142,59 @@
         <v>26</v>
       </c>
       <c r="B31" s="4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>Q1, Q2, Q3, Q4</t>
+          <t>R9, R28, R29, R30, R31, R32</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>BC337</t>
+          <t>10kΩ</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>THT</t>
+          <t>SMD</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>Package_TO_SOT_THT:TO-92_Inline</t>
+          <t>Resistor_SMD:R_0805_2012Metric</t>
         </is>
       </c>
       <c r="G31" s="4" t="inlineStr">
         <is>
-          <t>onsemi</t>
+          <t>YAGEO</t>
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr">
         <is>
-          <t>BC33740BU</t>
+          <t>RC0805FR-0710KL</t>
         </is>
       </c>
       <c r="I31" s="4" t="inlineStr">
         <is>
-          <t>512-BC33740BU</t>
+          <t>603-RC0805FR-0710KL</t>
         </is>
       </c>
       <c r="J31" s="7" t="n">
-        <v>0.249</v>
+        <v>0.08599999999999999</v>
       </c>
       <c r="K31" s="4" t="n">
-        <v>22995</v>
+        <v>3453672</v>
       </c>
       <c r="L31" s="4" t="inlineStr">
         <is>
-          <t>BC33740BU-ND</t>
+          <t>311-10.0KCRCT-ND</t>
         </is>
       </c>
       <c r="M31" s="6" t="n">
-        <v>0.25</v>
+        <v>0.09</v>
       </c>
       <c r="N31" s="4" t="n">
-        <v>2763</v>
+        <v>1935589</v>
       </c>
       <c r="O31" s="4" t="inlineStr">
         <is>
@@ -3241,26 +3241,26 @@
         <v>27</v>
       </c>
       <c r="B32" s="4" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>R9</t>
+          <t>R13, R15, R16, R33, R34</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>10k</t>
+          <t>220Ω</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>THT</t>
+          <t>SMD</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>Resistor_THT:R_Axial_DIN0207_L6.3mm_D2.5mm_P10.16mm_Horizontal</t>
+          <t>Resistor_SMD:R_0805_2012Metric</t>
         </is>
       </c>
       <c r="G32" s="4" t="inlineStr">
@@ -3270,30 +3270,30 @@
       </c>
       <c r="H32" s="4" t="inlineStr">
         <is>
-          <t>MFR-25FBF52-10K</t>
+          <t>RC0805FR-07220RL</t>
         </is>
       </c>
       <c r="I32" s="4" t="inlineStr">
         <is>
-          <t>603-MFR-25FBF52-10K</t>
+          <t>603-RC0805FR-07220RL</t>
         </is>
       </c>
       <c r="J32" s="7" t="n">
         <v>0.08599999999999999</v>
       </c>
       <c r="K32" s="4" t="n">
-        <v>128848</v>
+        <v>218894</v>
       </c>
       <c r="L32" s="4" t="inlineStr">
         <is>
-          <t>10.0KXBK-ND</t>
+          <t>311-220CRCT-ND</t>
         </is>
       </c>
       <c r="M32" s="6" t="n">
         <v>0.09</v>
       </c>
       <c r="N32" s="4" t="n">
-        <v>89882</v>
+        <v>380504</v>
       </c>
       <c r="O32" s="4" t="inlineStr">
         <is>
@@ -3340,59 +3340,59 @@
         <v>28</v>
       </c>
       <c r="B33" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>R13, R14, R15, R16</t>
+          <t>R14</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>220</t>
+          <t>100Ω</t>
         </is>
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>THT</t>
+          <t>SMD</t>
         </is>
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>Resistor_THT:R_Axial_DIN0617_L17.0mm_D6.0mm_P20.32mm_Horizontal</t>
+          <t>Resistor_SMD:R_0805_2012Metric</t>
         </is>
       </c>
       <c r="G33" s="4" t="inlineStr">
         <is>
-          <t>Vishay BC Components</t>
+          <t>YAGEO</t>
         </is>
       </c>
       <c r="H33" s="4" t="inlineStr">
         <is>
-          <t>PR02000202200JR500</t>
+          <t>RC0805FR-07100RL</t>
         </is>
       </c>
       <c r="I33" s="4" t="inlineStr">
         <is>
-          <t>594-5083NW220R0J</t>
-        </is>
-      </c>
-      <c r="J33" s="6" t="n">
-        <v>0.353</v>
+          <t>603-RC0805FR-07100RL</t>
+        </is>
+      </c>
+      <c r="J33" s="7" t="n">
+        <v>0.08599999999999999</v>
       </c>
       <c r="K33" s="4" t="n">
-        <v>4936</v>
+        <v>471173</v>
       </c>
       <c r="L33" s="4" t="inlineStr">
         <is>
-          <t>56-PR02000202200JR500CT-ND</t>
-        </is>
-      </c>
-      <c r="M33" s="7" t="n">
-        <v>0.35</v>
+          <t>311-100CRCT-ND</t>
+        </is>
+      </c>
+      <c r="M33" s="6" t="n">
+        <v>0.09</v>
       </c>
       <c r="N33" s="4" t="n">
-        <v>7451</v>
+        <v>1407631</v>
       </c>
       <c r="O33" s="4" t="inlineStr">
         <is>
@@ -3401,7 +3401,7 @@
       </c>
       <c r="P33" s="4" t="inlineStr">
         <is>
-          <t>DigiKey</t>
+          <t>Mouser</t>
         </is>
       </c>
       <c r="Q33" s="8">
@@ -3740,59 +3740,59 @@
         <v>32</v>
       </c>
       <c r="B37" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>R23, R24, R25, R26</t>
+          <t>R27</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>4,7k</t>
+          <t>12,4kΩ, 1%</t>
         </is>
       </c>
       <c r="E37" s="4" t="inlineStr">
         <is>
-          <t>THT</t>
+          <t>SMD</t>
         </is>
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>Resistor_THT:R_Axial_DIN0617_L17.0mm_D6.0mm_P20.32mm_Horizontal</t>
+          <t>Resistor_SMD:R_0805_2012Metric</t>
         </is>
       </c>
       <c r="G37" s="4" t="inlineStr">
         <is>
-          <t>Vishay BC Components</t>
+          <t>YAGEO</t>
         </is>
       </c>
       <c r="H37" s="4" t="inlineStr">
         <is>
-          <t>PR02000204701JR500</t>
+          <t>RC0805FR-0712K4L</t>
         </is>
       </c>
       <c r="I37" s="4" t="inlineStr">
         <is>
-          <t>594-5083NW4K700J</t>
-        </is>
-      </c>
-      <c r="J37" s="6" t="n">
-        <v>0.353</v>
+          <t>603-RC0805FR-0712K4L</t>
+        </is>
+      </c>
+      <c r="J37" s="7" t="n">
+        <v>0.08599999999999999</v>
       </c>
       <c r="K37" s="4" t="n">
-        <v>2586</v>
+        <v>9810</v>
       </c>
       <c r="L37" s="4" t="inlineStr">
         <is>
-          <t>56-PR02000204701JR500CT-ND</t>
-        </is>
-      </c>
-      <c r="M37" s="7" t="n">
-        <v>0.35</v>
+          <t>311-12.4KCRCT-ND</t>
+        </is>
+      </c>
+      <c r="M37" s="6" t="n">
+        <v>0.09</v>
       </c>
       <c r="N37" s="4" t="n">
-        <v>6005</v>
+        <v>13307</v>
       </c>
       <c r="O37" s="4" t="inlineStr">
         <is>
@@ -3801,7 +3801,7 @@
       </c>
       <c r="P37" s="4" t="inlineStr">
         <is>
-          <t>DigiKey</t>
+          <t>Mouser</t>
         </is>
       </c>
       <c r="Q37" s="8">
@@ -3843,12 +3843,12 @@
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>R27</t>
+          <t>R35</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>12,4kΩ, 1%</t>
+          <t>0Ω</t>
         </is>
       </c>
       <c r="E38" s="4" t="inlineStr">
@@ -3868,30 +3868,30 @@
       </c>
       <c r="H38" s="4" t="inlineStr">
         <is>
-          <t>RC0805FR-0712K4L</t>
+          <t>RC0805JR-070RL</t>
         </is>
       </c>
       <c r="I38" s="4" t="inlineStr">
         <is>
-          <t>603-RC0805FR-0712K4L</t>
-        </is>
-      </c>
-      <c r="J38" s="7" t="n">
-        <v>0.08599999999999999</v>
+          <t>603-RC0805JR-070RL</t>
+        </is>
+      </c>
+      <c r="J38" s="6" t="n">
+        <v>0.215</v>
       </c>
       <c r="K38" s="4" t="n">
-        <v>9810</v>
+        <v>2669469</v>
       </c>
       <c r="L38" s="4" t="inlineStr">
         <is>
-          <t>311-12.4KCRCT-ND</t>
-        </is>
-      </c>
-      <c r="M38" s="6" t="n">
+          <t>311-0.0ARCT-ND</t>
+        </is>
+      </c>
+      <c r="M38" s="7" t="n">
         <v>0.09</v>
       </c>
       <c r="N38" s="4" t="n">
-        <v>13307</v>
+        <v>2861448</v>
       </c>
       <c r="O38" s="4" t="inlineStr">
         <is>
@@ -3900,7 +3900,7 @@
       </c>
       <c r="P38" s="4" t="inlineStr">
         <is>
-          <t>Mouser</t>
+          <t>DigiKey</t>
         </is>
       </c>
       <c r="Q38" s="8">
@@ -3938,16 +3938,16 @@
         <v>34</v>
       </c>
       <c r="B39" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>R28, R29, R30, R31, R32</t>
+          <t>R36, R37, R39, R40</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>10kΩ</t>
+          <t>49,9Ω 1%</t>
         </is>
       </c>
       <c r="E39" s="4" t="inlineStr">
@@ -3967,30 +3967,30 @@
       </c>
       <c r="H39" s="4" t="inlineStr">
         <is>
-          <t>RC0805FR-0710KL</t>
+          <t>RC0805FR-0749R9L</t>
         </is>
       </c>
       <c r="I39" s="4" t="inlineStr">
         <is>
-          <t>603-RC0805FR-0710KL</t>
+          <t>603-RC0805FR-0749R9L</t>
         </is>
       </c>
       <c r="J39" s="7" t="n">
         <v>0.08599999999999999</v>
       </c>
       <c r="K39" s="4" t="n">
-        <v>3453672</v>
+        <v>308094</v>
       </c>
       <c r="L39" s="4" t="inlineStr">
         <is>
-          <t>311-10.0KCRCT-ND</t>
+          <t>311-49.9CRCT-ND</t>
         </is>
       </c>
       <c r="M39" s="6" t="n">
         <v>0.09</v>
       </c>
       <c r="N39" s="4" t="n">
-        <v>1935589</v>
+        <v>376340</v>
       </c>
       <c r="O39" s="4" t="inlineStr">
         <is>
@@ -4037,16 +4037,16 @@
         <v>35</v>
       </c>
       <c r="B40" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>R33, R34</t>
+          <t>R38</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>220Ω</t>
+          <t>10Ω 1%</t>
         </is>
       </c>
       <c r="E40" s="4" t="inlineStr">
@@ -4066,30 +4066,30 @@
       </c>
       <c r="H40" s="4" t="inlineStr">
         <is>
-          <t>RC0805FR-07220RL</t>
+          <t>RC0805FR-0710RL</t>
         </is>
       </c>
       <c r="I40" s="4" t="inlineStr">
         <is>
-          <t>603-RC0805FR-07220RL</t>
+          <t>603-RC0805FR-0710RL</t>
         </is>
       </c>
       <c r="J40" s="7" t="n">
         <v>0.08599999999999999</v>
       </c>
       <c r="K40" s="4" t="n">
-        <v>218894</v>
+        <v>119285</v>
       </c>
       <c r="L40" s="4" t="inlineStr">
         <is>
-          <t>311-220CRCT-ND</t>
+          <t>311-10.0CRCT-ND</t>
         </is>
       </c>
       <c r="M40" s="6" t="n">
-        <v>0.09</v>
+        <v>0.1</v>
       </c>
       <c r="N40" s="4" t="n">
-        <v>380504</v>
+        <v>601024</v>
       </c>
       <c r="O40" s="4" t="inlineStr">
         <is>
@@ -4140,55 +4140,55 @@
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>R35</t>
+          <t>S2</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>0Ω</t>
+          <t>PTS645VL58-2 LFS</t>
         </is>
       </c>
       <c r="E41" s="4" t="inlineStr">
         <is>
-          <t>SMD</t>
+          <t>THT</t>
         </is>
       </c>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>Resistor_SMD:R_0805_2012Metric</t>
+          <t>PTS645VL58-2LFS:SW_Tactile_SPST_Angled_PTS645Vx58-2LFS</t>
         </is>
       </c>
       <c r="G41" s="4" t="inlineStr">
         <is>
-          <t>YAGEO</t>
+          <t>C&amp;K</t>
         </is>
       </c>
       <c r="H41" s="4" t="inlineStr">
         <is>
-          <t>RC0805JR-070RL</t>
+          <t>PTS645VL58-2 LFS</t>
         </is>
       </c>
       <c r="I41" s="4" t="inlineStr">
         <is>
-          <t>603-RC0805JR-070RL</t>
-        </is>
-      </c>
-      <c r="J41" s="6" t="n">
-        <v>0.215</v>
+          <t>611-PTS645VL582</t>
+        </is>
+      </c>
+      <c r="J41" s="7" t="n">
+        <v>0.284</v>
       </c>
       <c r="K41" s="4" t="n">
-        <v>2669469</v>
+        <v>290</v>
       </c>
       <c r="L41" s="4" t="inlineStr">
         <is>
-          <t>311-0.0ARCT-ND</t>
-        </is>
-      </c>
-      <c r="M41" s="7" t="n">
-        <v>0.09</v>
+          <t>CKN9116-ND</t>
+        </is>
+      </c>
+      <c r="M41" s="6" t="n">
+        <v>0.36</v>
       </c>
       <c r="N41" s="4" t="n">
-        <v>2861448</v>
+        <v>19085</v>
       </c>
       <c r="O41" s="4" t="inlineStr">
         <is>
@@ -4197,7 +4197,7 @@
       </c>
       <c r="P41" s="4" t="inlineStr">
         <is>
-          <t>DigiKey</t>
+          <t>Mouser</t>
         </is>
       </c>
       <c r="Q41" s="8">
@@ -4235,59 +4235,59 @@
         <v>37</v>
       </c>
       <c r="B42" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>R36, R37, R39, R40</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>49,9Ω 1%</t>
+          <t>7499011121A</t>
         </is>
       </c>
       <c r="E42" s="4" t="inlineStr">
         <is>
-          <t>SMD</t>
+          <t>THT</t>
         </is>
       </c>
       <c r="F42" s="4" t="inlineStr">
         <is>
-          <t>Resistor_SMD:R_0805_2012Metric</t>
+          <t>wuerth_rj45:T_Wurth_WE-RJ45LAN_7499011121A</t>
         </is>
       </c>
       <c r="G42" s="4" t="inlineStr">
         <is>
-          <t>YAGEO</t>
+          <t>Wurth Elektronik</t>
         </is>
       </c>
       <c r="H42" s="4" t="inlineStr">
         <is>
-          <t>RC0805FR-0749R9L</t>
+          <t>7499011121A</t>
         </is>
       </c>
       <c r="I42" s="4" t="inlineStr">
         <is>
-          <t>603-RC0805FR-0749R9L</t>
-        </is>
-      </c>
-      <c r="J42" s="7" t="n">
-        <v>0.08599999999999999</v>
+          <t>710-7499011121A</t>
+        </is>
+      </c>
+      <c r="J42" s="6" t="n">
+        <v>6.26</v>
       </c>
       <c r="K42" s="4" t="n">
-        <v>308094</v>
+        <v>1259</v>
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>311-49.9CRCT-ND</t>
-        </is>
-      </c>
-      <c r="M42" s="6" t="n">
-        <v>0.09</v>
+          <t>732-4509-5-ND</t>
+        </is>
+      </c>
+      <c r="M42" s="7" t="n">
+        <v>5.92</v>
       </c>
       <c r="N42" s="4" t="n">
-        <v>376340</v>
+        <v>2673</v>
       </c>
       <c r="O42" s="4" t="inlineStr">
         <is>
@@ -4296,7 +4296,7 @@
       </c>
       <c r="P42" s="4" t="inlineStr">
         <is>
-          <t>Mouser</t>
+          <t>DigiKey</t>
         </is>
       </c>
       <c r="Q42" s="8">
@@ -4338,12 +4338,12 @@
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>R38</t>
+          <t>U1</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t>10Ω 1%</t>
+          <t>D3V3XA4B10LP</t>
         </is>
       </c>
       <c r="E43" s="4" t="inlineStr">
@@ -4353,40 +4353,40 @@
       </c>
       <c r="F43" s="4" t="inlineStr">
         <is>
-          <t>Resistor_SMD:R_0805_2012Metric</t>
+          <t>Package_DFN_QFN:Diodes_UDFN-10_1x2.5mm_P0.5mm</t>
         </is>
       </c>
       <c r="G43" s="4" t="inlineStr">
         <is>
-          <t>YAGEO</t>
+          <t>Diodes Incorporated</t>
         </is>
       </c>
       <c r="H43" s="4" t="inlineStr">
         <is>
-          <t>RC0805FR-0710RL</t>
+          <t>D3V3XA4B10LP-7</t>
         </is>
       </c>
       <c r="I43" s="4" t="inlineStr">
         <is>
-          <t>603-RC0805FR-0710RL</t>
+          <t>621-D3V3XA4B10LP-7</t>
         </is>
       </c>
       <c r="J43" s="7" t="n">
-        <v>0.08599999999999999</v>
+        <v>0.37</v>
       </c>
       <c r="K43" s="4" t="n">
-        <v>119285</v>
+        <v>11929</v>
       </c>
       <c r="L43" s="4" t="inlineStr">
         <is>
-          <t>311-10.0CRCT-ND</t>
+          <t>31-D3V3XA4B10LP-7CT-ND</t>
         </is>
       </c>
       <c r="M43" s="6" t="n">
-        <v>0.1</v>
+        <v>0.39</v>
       </c>
       <c r="N43" s="4" t="n">
-        <v>601024</v>
+        <v>11467</v>
       </c>
       <c r="O43" s="4" t="inlineStr">
         <is>
@@ -4437,55 +4437,55 @@
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>S2</t>
+          <t>U6</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>PTS645VL58-2 LFS</t>
+          <t>ESP32-S3-WROOM-1U-N16R8</t>
         </is>
       </c>
       <c r="E44" s="4" t="inlineStr">
         <is>
-          <t>THT</t>
+          <t>SMD</t>
         </is>
       </c>
       <c r="F44" s="4" t="inlineStr">
         <is>
-          <t>PTS645VL58-2LFS:SW_Tactile_SPST_Angled_PTS645Vx58-2LFS</t>
+          <t>ESP32-S3-WROOM-1U-N16R8:ESP32-S3-WROOM-1U</t>
         </is>
       </c>
       <c r="G44" s="4" t="inlineStr">
         <is>
-          <t>C&amp;K</t>
+          <t>Espressif Systems</t>
         </is>
       </c>
       <c r="H44" s="4" t="inlineStr">
         <is>
-          <t>PTS645VL58-2 LFS</t>
+          <t>ESP32-S3-WROOM-1U-N16R8</t>
         </is>
       </c>
       <c r="I44" s="4" t="inlineStr">
         <is>
-          <t>611-PTS645VL582</t>
-        </is>
-      </c>
-      <c r="J44" s="7" t="n">
-        <v>0.284</v>
+          <t>356-ESP32S3WM1UN16R8</t>
+        </is>
+      </c>
+      <c r="J44" s="6" t="n">
+        <v>5.93</v>
       </c>
       <c r="K44" s="4" t="n">
-        <v>290</v>
+        <v>6109</v>
       </c>
       <c r="L44" s="4" t="inlineStr">
         <is>
-          <t>CKN9116-ND</t>
-        </is>
-      </c>
-      <c r="M44" s="6" t="n">
-        <v>0.36</v>
+          <t>1965-ESP32-S3-WROOM-1U-N16R8CT-ND</t>
+        </is>
+      </c>
+      <c r="M44" s="7" t="n">
+        <v>5.79</v>
       </c>
       <c r="N44" s="4" t="n">
-        <v>19085</v>
+        <v>66</v>
       </c>
       <c r="O44" s="4" t="inlineStr">
         <is>
@@ -4525,7 +4525,11 @@
           <t>eindeutig</t>
         </is>
       </c>
-      <c r="W44" s="5" t="inlineStr"/>
+      <c r="W44" s="5" t="inlineStr">
+        <is>
+          <t>Bezugsquelle Mouser festgelegt (Bediener, 2026-09-24): DigiKey hat nur zweistelligen Lagerbestand, Mouser mehrere Tausend — sicherer fuer groessere Stueckzahlen, Aufpreis rund 0,14 EUR.</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="4" t="n">
@@ -4536,55 +4540,55 @@
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>U7</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>7499011121A</t>
+          <t>W5500</t>
         </is>
       </c>
       <c r="E45" s="4" t="inlineStr">
         <is>
-          <t>THT</t>
+          <t>SMD</t>
         </is>
       </c>
       <c r="F45" s="4" t="inlineStr">
         <is>
-          <t>wuerth_rj45:T_Wurth_WE-RJ45LAN_7499011121A</t>
+          <t>W5500:48LQFP_W5500_WIZ</t>
         </is>
       </c>
       <c r="G45" s="4" t="inlineStr">
         <is>
-          <t>Wurth Elektronik</t>
+          <t>WIZnet</t>
         </is>
       </c>
       <c r="H45" s="4" t="inlineStr">
         <is>
-          <t>7499011121A</t>
+          <t>W5500</t>
         </is>
       </c>
       <c r="I45" s="4" t="inlineStr">
         <is>
-          <t>710-7499011121A</t>
-        </is>
-      </c>
-      <c r="J45" s="6" t="n">
-        <v>6.26</v>
+          <t>950-W5500</t>
+        </is>
+      </c>
+      <c r="J45" s="7" t="n">
+        <v>2.98</v>
       </c>
       <c r="K45" s="4" t="n">
-        <v>1259</v>
+        <v>43173</v>
       </c>
       <c r="L45" s="4" t="inlineStr">
         <is>
-          <t>732-4509-5-ND</t>
-        </is>
-      </c>
-      <c r="M45" s="7" t="n">
-        <v>5.92</v>
+          <t>1278-W5500CT-ND</t>
+        </is>
+      </c>
+      <c r="M45" s="6" t="n">
+        <v>3.18</v>
       </c>
       <c r="N45" s="4" t="n">
-        <v>2673</v>
+        <v>62550</v>
       </c>
       <c r="O45" s="4" t="inlineStr">
         <is>
@@ -4593,7 +4597,7 @@
       </c>
       <c r="P45" s="4" t="inlineStr">
         <is>
-          <t>DigiKey</t>
+          <t>Mouser</t>
         </is>
       </c>
       <c r="Q45" s="8">
@@ -4635,12 +4639,12 @@
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>U1</t>
+          <t>Y1</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t>D3V3XA4B10LP</t>
+          <t>25 MHz</t>
         </is>
       </c>
       <c r="E46" s="4" t="inlineStr">
@@ -4650,40 +4654,40 @@
       </c>
       <c r="F46" s="4" t="inlineStr">
         <is>
-          <t>Package_DFN_QFN:Diodes_UDFN-10_1x2.5mm_P0.5mm</t>
+          <t>wuerth_830059532:Y_Wurth_WE-XTAL_Quartz-CFPX-104</t>
         </is>
       </c>
       <c r="G46" s="4" t="inlineStr">
         <is>
-          <t>Diodes Incorporated</t>
+          <t>Wurth Elektronik</t>
         </is>
       </c>
       <c r="H46" s="4" t="inlineStr">
         <is>
-          <t>D3V3XA4B10LP-7</t>
+          <t>830059532</t>
         </is>
       </c>
       <c r="I46" s="4" t="inlineStr">
         <is>
-          <t>621-D3V3XA4B10LP-7</t>
-        </is>
-      </c>
-      <c r="J46" s="7" t="n">
-        <v>0.37</v>
+          <t>710-830059532</t>
+        </is>
+      </c>
+      <c r="J46" s="6" t="n">
+        <v>0.757</v>
       </c>
       <c r="K46" s="4" t="n">
-        <v>11929</v>
+        <v>3563</v>
       </c>
       <c r="L46" s="4" t="inlineStr">
         <is>
-          <t>31-D3V3XA4B10LP-7CT-ND</t>
-        </is>
-      </c>
-      <c r="M46" s="6" t="n">
-        <v>0.39</v>
+          <t>1923-830059532CT-ND</t>
+        </is>
+      </c>
+      <c r="M46" s="7" t="n">
+        <v>0.75</v>
       </c>
       <c r="N46" s="4" t="n">
-        <v>11467</v>
+        <v>3667</v>
       </c>
       <c r="O46" s="4" t="inlineStr">
         <is>
@@ -4692,7 +4696,7 @@
       </c>
       <c r="P46" s="4" t="inlineStr">
         <is>
-          <t>Mouser</t>
+          <t>DigiKey</t>
         </is>
       </c>
       <c r="Q46" s="8">
@@ -4725,351 +4729,50 @@
       </c>
       <c r="W46" s="5" t="inlineStr"/>
     </row>
-    <row r="47">
-      <c r="A47" s="4" t="n">
-        <v>42</v>
-      </c>
-      <c r="B47" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="C47" s="5" t="inlineStr">
-        <is>
-          <t>U6</t>
-        </is>
-      </c>
-      <c r="D47" s="4" t="inlineStr">
-        <is>
-          <t>ESP32-S3-WROOM-1U-N16R8</t>
-        </is>
-      </c>
-      <c r="E47" s="4" t="inlineStr">
-        <is>
-          <t>SMD</t>
-        </is>
-      </c>
-      <c r="F47" s="4" t="inlineStr">
-        <is>
-          <t>ESP32-S3-WROOM-1U-N16R8:ESP32-S3-WROOM-1U</t>
-        </is>
-      </c>
-      <c r="G47" s="4" t="inlineStr">
-        <is>
-          <t>Espressif Systems</t>
-        </is>
-      </c>
-      <c r="H47" s="4" t="inlineStr">
-        <is>
-          <t>ESP32-S3-WROOM-1U-N16R8</t>
-        </is>
-      </c>
-      <c r="I47" s="4" t="inlineStr">
-        <is>
-          <t>356-ESP32S3WM1UN16R8</t>
-        </is>
-      </c>
-      <c r="J47" s="6" t="n">
-        <v>5.93</v>
-      </c>
-      <c r="K47" s="4" t="n">
-        <v>6109</v>
-      </c>
-      <c r="L47" s="4" t="inlineStr">
-        <is>
-          <t>1965-ESP32-S3-WROOM-1U-N16R8CT-ND</t>
-        </is>
-      </c>
-      <c r="M47" s="7" t="n">
-        <v>5.79</v>
-      </c>
-      <c r="N47" s="4" t="n">
-        <v>66</v>
-      </c>
-      <c r="O47" s="4" t="inlineStr">
-        <is>
-          <t>Aktiv</t>
-        </is>
-      </c>
-      <c r="P47" s="4" t="inlineStr">
-        <is>
-          <t>Mouser</t>
-        </is>
-      </c>
-      <c r="Q47" s="8">
-        <f>IF(P47="DigiKey",IF(M47="","",M47),IF(P47="Mouser",IF(J47="","",J47),""))</f>
+    <row r="48">
+      <c r="P48" s="11" t="inlineStr">
+        <is>
+          <t>Summe erfasster Positionen</t>
+        </is>
+      </c>
+      <c r="R48" s="12">
+        <f>SUM(R6:R46)</f>
         <v/>
       </c>
-      <c r="R47" s="8">
-        <f>IF(OR(Q47="",B47=""),"",B47*Q47)</f>
+    </row>
+    <row r="49">
+      <c r="P49" s="13" t="inlineStr">
+        <is>
+          <t>davon DigiKey</t>
+        </is>
+      </c>
+      <c r="R49" s="14">
+        <f>SUMIF(P6:P46,"DigiKey",R6:R46)</f>
         <v/>
       </c>
-      <c r="S47" s="9" t="inlineStr">
-        <is>
-          <t>Mouser</t>
-        </is>
-      </c>
-      <c r="T47" s="9" t="inlineStr">
-        <is>
-          <t>DigiKey</t>
-        </is>
-      </c>
-      <c r="U47" s="9" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
-      <c r="V47" s="4" t="inlineStr">
-        <is>
-          <t>eindeutig</t>
-        </is>
-      </c>
-      <c r="W47" s="5" t="inlineStr">
-        <is>
-          <t>Bezugsquelle Mouser festgelegt (Bediener, 2026-09-24): DigiKey hat nur zweistelligen Lagerbestand, Mouser mehrere Tausend — sicherer fuer groessere Stueckzahlen, Aufpreis rund 0,14 EUR.</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="4" t="n">
-        <v>43</v>
-      </c>
-      <c r="B48" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="C48" s="5" t="inlineStr">
-        <is>
-          <t>U7</t>
-        </is>
-      </c>
-      <c r="D48" s="4" t="inlineStr">
-        <is>
-          <t>W5500</t>
-        </is>
-      </c>
-      <c r="E48" s="4" t="inlineStr">
-        <is>
-          <t>SMD</t>
-        </is>
-      </c>
-      <c r="F48" s="4" t="inlineStr">
-        <is>
-          <t>W5500:48LQFP_W5500_WIZ</t>
-        </is>
-      </c>
-      <c r="G48" s="4" t="inlineStr">
-        <is>
-          <t>WIZnet</t>
-        </is>
-      </c>
-      <c r="H48" s="4" t="inlineStr">
-        <is>
-          <t>W5500</t>
-        </is>
-      </c>
-      <c r="I48" s="4" t="inlineStr">
-        <is>
-          <t>950-W5500</t>
-        </is>
-      </c>
-      <c r="J48" s="7" t="n">
-        <v>2.98</v>
-      </c>
-      <c r="K48" s="4" t="n">
-        <v>43173</v>
-      </c>
-      <c r="L48" s="4" t="inlineStr">
-        <is>
-          <t>1278-W5500CT-ND</t>
-        </is>
-      </c>
-      <c r="M48" s="6" t="n">
-        <v>3.18</v>
-      </c>
-      <c r="N48" s="4" t="n">
-        <v>62550</v>
-      </c>
-      <c r="O48" s="4" t="inlineStr">
-        <is>
-          <t>Aktiv</t>
-        </is>
-      </c>
-      <c r="P48" s="4" t="inlineStr">
-        <is>
-          <t>Mouser</t>
-        </is>
-      </c>
-      <c r="Q48" s="8">
-        <f>IF(P48="DigiKey",IF(M48="","",M48),IF(P48="Mouser",IF(J48="","",J48),""))</f>
+    </row>
+    <row r="50">
+      <c r="P50" s="13" t="inlineStr">
+        <is>
+          <t>davon Mouser</t>
+        </is>
+      </c>
+      <c r="R50" s="14">
+        <f>SUMIF(P6:P46,"Mouser",R6:R46)</f>
         <v/>
       </c>
-      <c r="R48" s="8">
-        <f>IF(OR(Q48="",B48=""),"",B48*Q48)</f>
-        <v/>
-      </c>
-      <c r="S48" s="9" t="inlineStr">
-        <is>
-          <t>Mouser</t>
-        </is>
-      </c>
-      <c r="T48" s="9" t="inlineStr">
-        <is>
-          <t>DigiKey</t>
-        </is>
-      </c>
-      <c r="U48" s="9" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
-      <c r="V48" s="4" t="inlineStr">
-        <is>
-          <t>eindeutig</t>
-        </is>
-      </c>
-      <c r="W48" s="5" t="inlineStr"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="4" t="n">
-        <v>44</v>
-      </c>
-      <c r="B49" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="C49" s="5" t="inlineStr">
-        <is>
-          <t>Y1</t>
-        </is>
-      </c>
-      <c r="D49" s="4" t="inlineStr">
-        <is>
-          <t>25 MHz</t>
-        </is>
-      </c>
-      <c r="E49" s="4" t="inlineStr">
-        <is>
-          <t>SMD</t>
-        </is>
-      </c>
-      <c r="F49" s="4" t="inlineStr">
-        <is>
-          <t>wuerth_830059532:Y_Wurth_WE-XTAL_Quartz-CFPX-104</t>
-        </is>
-      </c>
-      <c r="G49" s="4" t="inlineStr">
-        <is>
-          <t>Wurth Elektronik</t>
-        </is>
-      </c>
-      <c r="H49" s="4" t="inlineStr">
-        <is>
-          <t>830059532</t>
-        </is>
-      </c>
-      <c r="I49" s="4" t="inlineStr">
-        <is>
-          <t>710-830059532</t>
-        </is>
-      </c>
-      <c r="J49" s="6" t="n">
-        <v>0.757</v>
-      </c>
-      <c r="K49" s="4" t="n">
-        <v>3563</v>
-      </c>
-      <c r="L49" s="4" t="inlineStr">
-        <is>
-          <t>1923-830059532CT-ND</t>
-        </is>
-      </c>
-      <c r="M49" s="7" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="N49" s="4" t="n">
-        <v>3667</v>
-      </c>
-      <c r="O49" s="4" t="inlineStr">
-        <is>
-          <t>Aktiv</t>
-        </is>
-      </c>
-      <c r="P49" s="4" t="inlineStr">
-        <is>
-          <t>DigiKey</t>
-        </is>
-      </c>
-      <c r="Q49" s="8">
-        <f>IF(P49="DigiKey",IF(M49="","",M49),IF(P49="Mouser",IF(J49="","",J49),""))</f>
-        <v/>
-      </c>
-      <c r="R49" s="8">
-        <f>IF(OR(Q49="",B49=""),"",B49*Q49)</f>
-        <v/>
-      </c>
-      <c r="S49" s="9" t="inlineStr">
-        <is>
-          <t>Mouser</t>
-        </is>
-      </c>
-      <c r="T49" s="9" t="inlineStr">
-        <is>
-          <t>DigiKey</t>
-        </is>
-      </c>
-      <c r="U49" s="9" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
-      <c r="V49" s="4" t="inlineStr">
-        <is>
-          <t>eindeutig</t>
-        </is>
-      </c>
-      <c r="W49" s="5" t="inlineStr"/>
-    </row>
-    <row r="51">
-      <c r="P51" s="11" t="inlineStr">
-        <is>
-          <t>Summe erfasster Positionen</t>
-        </is>
-      </c>
-      <c r="R51" s="12">
-        <f>SUM(R6:R49)</f>
-        <v/>
-      </c>
     </row>
     <row r="52">
-      <c r="P52" s="13" t="inlineStr">
-        <is>
-          <t>davon DigiKey</t>
-        </is>
-      </c>
-      <c r="R52" s="14">
-        <f>SUMIF(P6:P49,"DigiKey",R6:R49)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="53">
-      <c r="P53" s="13" t="inlineStr">
-        <is>
-          <t>davon Mouser</t>
-        </is>
-      </c>
-      <c r="R53" s="14">
-        <f>SUMIF(P6:P49,"Mouser",R6:R49)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Von 44 Positionen tragen 44 einen Preis aus der API (18 über DigiKey, 26 über Mouser). </t>
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Von 41 Positionen tragen 41 einen Preis aus der API (16 über DigiKey, 25 über Mouser). </t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A5:W49"/>
+  <autoFilter ref="A5:W46"/>
   <dataValidations count="1">
-    <dataValidation sqref="P6 P7 P8 P9 P10 P11 P12 P13 P14 P15 P16 P17 P18 P19 P20 P21 P22 P23 P24 P25 P26 P27 P28 P29 P30 P31 P32 P33 P34 P35 P36 P37 P38 P39 P40 P41 P42 P43 P44 P45 P46 P47 P48 P49" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="P6 P7 P8 P9 P10 P11 P12 P13 P14 P15 P16 P17 P18 P19 P20 P21 P22 P23 P24 P25 P26 P27 P28 P29 P30 P31 P32 P33 P34 P35 P36 P37 P38 P39 P40 P41 P42 P43 P44 P45 P46" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"DigiKey,Mouser"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5197,15 +4900,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S46" r:id="rId121"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T46" r:id="rId122"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U46" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S47" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T47" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U47" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S48" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T48" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U48" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S49" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T49" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U49" r:id="rId132"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5217,7 +4911,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I83"/>
+  <dimension ref="A1:I75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5241,7 +4935,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Alle 78 bestückten Referenzen einzeln · Stand 2026-09-29</t>
+          <t>Alle 70 bestückten Referenzen einzeln · Stand 2026-09-30</t>
         </is>
       </c>
     </row>
@@ -5369,7 +5063,7 @@
       </c>
       <c r="E7" s="15" t="inlineStr">
         <is>
-          <t>Connector:USB_C_Receptacle_USB2.0_16P</t>
+          <t>shbs_power:USB_C_Receptacle_USB2.0_16P</t>
         </is>
       </c>
       <c r="F7" s="15" t="inlineStr">
@@ -5490,19 +5184,15 @@
     <row r="10">
       <c r="A10" s="15" t="inlineStr">
         <is>
-          <t>Q1</t>
+          <t>ANT2</t>
         </is>
       </c>
       <c r="B10" s="15" t="inlineStr">
         <is>
-          <t>BC337</t>
-        </is>
-      </c>
-      <c r="C10" s="15" t="inlineStr">
-        <is>
-          <t>THT</t>
-        </is>
-      </c>
+          <t>GW.20.A151</t>
+        </is>
+      </c>
+      <c r="C10" s="15" t="inlineStr"/>
       <c r="D10" s="15" t="inlineStr">
         <is>
           <t>BasisStation_Layout.kicad_sch</t>
@@ -5510,42 +5200,42 @@
       </c>
       <c r="E10" s="15" t="inlineStr">
         <is>
-          <t>Transistor_BJT:BC337</t>
-        </is>
-      </c>
-      <c r="F10" s="15" t="inlineStr">
-        <is>
-          <t>Package_TO_SOT_THT:TO-92_Inline</t>
-        </is>
-      </c>
+          <t>mechanical:WLAN_Antenna</t>
+        </is>
+      </c>
+      <c r="F10" s="15" t="inlineStr"/>
       <c r="G10" s="15" t="inlineStr">
         <is>
-          <t>onsemi</t>
+          <t>Taoglas</t>
         </is>
       </c>
       <c r="H10" s="15" t="inlineStr">
         <is>
-          <t>BC33740BU</t>
+          <t>GW.20.A151</t>
         </is>
       </c>
       <c r="I10" s="15" t="inlineStr">
         <is>
-          <t>512-BC33740BU</t>
+          <t>960-GW.20.A151</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="15" t="inlineStr">
         <is>
-          <t>ANT2</t>
+          <t>D9</t>
         </is>
       </c>
       <c r="B11" s="15" t="inlineStr">
         <is>
-          <t>GW.20.A151</t>
-        </is>
-      </c>
-      <c r="C11" s="15" t="inlineStr"/>
+          <t>RED</t>
+        </is>
+      </c>
+      <c r="C11" s="15" t="inlineStr">
+        <is>
+          <t>SMD</t>
+        </is>
+      </c>
       <c r="D11" s="15" t="inlineStr">
         <is>
           <t>BasisStation_Layout.kicad_sch</t>
@@ -5553,42 +5243,42 @@
       </c>
       <c r="E11" s="15" t="inlineStr">
         <is>
-          <t>mechanical:WLAN_Antenna</t>
-        </is>
-      </c>
-      <c r="F11" s="15" t="inlineStr"/>
+          <t>Device:LED</t>
+        </is>
+      </c>
+      <c r="F11" s="15" t="inlineStr">
+        <is>
+          <t>LED_THT:LED_D3.0mm_Horizontal_O1.27mm_Z2.0mm</t>
+        </is>
+      </c>
       <c r="G11" s="15" t="inlineStr">
         <is>
-          <t>Taoglas</t>
+          <t>Würth Elektronik</t>
         </is>
       </c>
       <c r="H11" s="15" t="inlineStr">
         <is>
-          <t>GW.20.A151</t>
+          <t>151033RS03000</t>
         </is>
       </c>
       <c r="I11" s="15" t="inlineStr">
         <is>
-          <t>960-GW.20.A151</t>
+          <t>710-151033RS03000</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="15" t="inlineStr">
         <is>
-          <t>D9</t>
+          <t>ANT1</t>
         </is>
       </c>
       <c r="B12" s="15" t="inlineStr">
         <is>
-          <t>RED</t>
-        </is>
-      </c>
-      <c r="C12" s="15" t="inlineStr">
-        <is>
-          <t>THT</t>
-        </is>
-      </c>
+          <t>CAB.6061</t>
+        </is>
+      </c>
+      <c r="C12" s="15" t="inlineStr"/>
       <c r="D12" s="15" t="inlineStr">
         <is>
           <t>BasisStation_Layout.kicad_sch</t>
@@ -5596,42 +5286,42 @@
       </c>
       <c r="E12" s="15" t="inlineStr">
         <is>
-          <t>Device:LED</t>
-        </is>
-      </c>
-      <c r="F12" s="15" t="inlineStr">
-        <is>
-          <t>WL-TMRW_3MM:WL-TMRW_3MM</t>
-        </is>
-      </c>
+          <t>mechanical:WLAN_Pigtail</t>
+        </is>
+      </c>
+      <c r="F12" s="15" t="inlineStr"/>
       <c r="G12" s="15" t="inlineStr">
         <is>
-          <t>Würth Elektronik</t>
+          <t>Taoglas</t>
         </is>
       </c>
       <c r="H12" s="15" t="inlineStr">
         <is>
-          <t>151033RS03000</t>
+          <t>CAB.6061</t>
         </is>
       </c>
       <c r="I12" s="15" t="inlineStr">
         <is>
-          <t>710-151033RS03000</t>
+          <t>960-CAB.6061</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="15" t="inlineStr">
         <is>
-          <t>ANT1</t>
+          <t>C10</t>
         </is>
       </c>
       <c r="B13" s="15" t="inlineStr">
         <is>
-          <t>CAB.6061</t>
-        </is>
-      </c>
-      <c r="C13" s="15" t="inlineStr"/>
+          <t>WCAP-FTXX_P10</t>
+        </is>
+      </c>
+      <c r="C13" s="15" t="inlineStr">
+        <is>
+          <t>SMD</t>
+        </is>
+      </c>
       <c r="D13" s="15" t="inlineStr">
         <is>
           <t>BasisStation_Layout.kicad_sch</t>
@@ -5639,35 +5329,35 @@
       </c>
       <c r="E13" s="15" t="inlineStr">
         <is>
-          <t>mechanical:WLAN_Pigtail</t>
-        </is>
-      </c>
-      <c r="F13" s="15" t="inlineStr"/>
+          <t>WCAP-FTXX_P10:WCAP-FTXX_P10</t>
+        </is>
+      </c>
+      <c r="F13" s="15" t="inlineStr">
+        <is>
+          <t>WCAP-FTXX_P10:WCAP-FTXX_P10L13W7H13</t>
+        </is>
+      </c>
       <c r="G13" s="15" t="inlineStr">
         <is>
-          <t>Taoglas</t>
+          <t>Würth Elektronik</t>
         </is>
       </c>
       <c r="H13" s="15" t="inlineStr">
         <is>
-          <t>CAB.6061</t>
-        </is>
-      </c>
-      <c r="I13" s="15" t="inlineStr">
-        <is>
-          <t>960-CAB.6061</t>
-        </is>
-      </c>
+          <t>890334023023</t>
+        </is>
+      </c>
+      <c r="I13" s="15" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="15" t="inlineStr">
         <is>
-          <t>C10</t>
+          <t>D7</t>
         </is>
       </c>
       <c r="B14" s="15" t="inlineStr">
         <is>
-          <t>WCAP-FTXX_P10</t>
+          <t>YELLOW</t>
         </is>
       </c>
       <c r="C14" s="15" t="inlineStr">
@@ -5682,22 +5372,22 @@
       </c>
       <c r="E14" s="15" t="inlineStr">
         <is>
-          <t>WCAP-FTXX_P10:WCAP-FTXX_P10</t>
+          <t>Device:LED</t>
         </is>
       </c>
       <c r="F14" s="15" t="inlineStr">
         <is>
-          <t>WCAP-FTXX_P10:WCAP-FTXX_P10L13W7H13</t>
+          <t>LED_THT:LED_D3.0mm_Horizontal_O1.27mm_Z2.0mm</t>
         </is>
       </c>
       <c r="G14" s="15" t="inlineStr">
         <is>
-          <t>Würth Elektronik</t>
+          <t>Wurth Electronics</t>
         </is>
       </c>
       <c r="H14" s="15" t="inlineStr">
         <is>
-          <t>890334023023</t>
+          <t>151031YS05900</t>
         </is>
       </c>
       <c r="I14" s="15" t="inlineStr"/>
@@ -5705,17 +5395,17 @@
     <row r="15">
       <c r="A15" s="15" t="inlineStr">
         <is>
-          <t>D7</t>
+          <t>R14</t>
         </is>
       </c>
       <c r="B15" s="15" t="inlineStr">
         <is>
-          <t>YELLOW</t>
+          <t>100Ω</t>
         </is>
       </c>
       <c r="C15" s="15" t="inlineStr">
         <is>
-          <t>THT</t>
+          <t>SMD</t>
         </is>
       </c>
       <c r="D15" s="15" t="inlineStr">
@@ -5725,40 +5415,44 @@
       </c>
       <c r="E15" s="15" t="inlineStr">
         <is>
-          <t>Device:LED</t>
+          <t>Device:R</t>
         </is>
       </c>
       <c r="F15" s="15" t="inlineStr">
         <is>
-          <t>WL-TMRC_3MM:WL-TMRC_3MM</t>
+          <t>Resistor_SMD:R_0805_2012Metric</t>
         </is>
       </c>
       <c r="G15" s="15" t="inlineStr">
         <is>
-          <t>Wurth Electronics</t>
+          <t>YAGEO</t>
         </is>
       </c>
       <c r="H15" s="15" t="inlineStr">
         <is>
-          <t>151031YS05900</t>
-        </is>
-      </c>
-      <c r="I15" s="15" t="inlineStr"/>
+          <t>RC0805FR-07100RL</t>
+        </is>
+      </c>
+      <c r="I15" s="15" t="inlineStr">
+        <is>
+          <t>603-RC0805FR-07100RL</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="15" t="inlineStr">
         <is>
-          <t>R14</t>
+          <t>R15</t>
         </is>
       </c>
       <c r="B16" s="15" t="inlineStr">
         <is>
-          <t>220</t>
+          <t>220Ω</t>
         </is>
       </c>
       <c r="C16" s="15" t="inlineStr">
         <is>
-          <t>THT</t>
+          <t>SMD</t>
         </is>
       </c>
       <c r="D16" s="15" t="inlineStr">
@@ -5773,39 +5467,39 @@
       </c>
       <c r="F16" s="15" t="inlineStr">
         <is>
-          <t>Resistor_THT:R_Axial_DIN0617_L17.0mm_D6.0mm_P20.32mm_Horizontal</t>
+          <t>Resistor_SMD:R_0805_2012Metric</t>
         </is>
       </c>
       <c r="G16" s="15" t="inlineStr">
         <is>
-          <t>Vishay BC Components</t>
+          <t>YAGEO</t>
         </is>
       </c>
       <c r="H16" s="15" t="inlineStr">
         <is>
-          <t>PR02000202200JR500</t>
+          <t>RC0805FR-07220RL</t>
         </is>
       </c>
       <c r="I16" s="15" t="inlineStr">
         <is>
-          <t>594-5083NW220R0J</t>
+          <t>603-RC0805FR-07220RL</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="15" t="inlineStr">
         <is>
-          <t>Q4</t>
+          <t>C8</t>
         </is>
       </c>
       <c r="B17" s="15" t="inlineStr">
         <is>
-          <t>BC337</t>
+          <t>WCAP-PT5H_6.3X5.2</t>
         </is>
       </c>
       <c r="C17" s="15" t="inlineStr">
         <is>
-          <t>THT</t>
+          <t>SMD</t>
         </is>
       </c>
       <c r="D17" s="15" t="inlineStr">
@@ -5815,44 +5509,40 @@
       </c>
       <c r="E17" s="15" t="inlineStr">
         <is>
-          <t>Transistor_BJT:BC337</t>
+          <t>WCAP-PT5H_6.3X5.2:WCAP-PT5H_6.3X5.2</t>
         </is>
       </c>
       <c r="F17" s="15" t="inlineStr">
         <is>
-          <t>Package_TO_SOT_THT:TO-92_Inline</t>
+          <t>WCAP-PT5H_6.3X5.2:WCAP-PT5H_6.3X5.2_DXL_</t>
         </is>
       </c>
       <c r="G17" s="15" t="inlineStr">
         <is>
-          <t>onsemi</t>
+          <t>Wurth Elektronik</t>
         </is>
       </c>
       <c r="H17" s="15" t="inlineStr">
         <is>
-          <t>BC33740BU</t>
-        </is>
-      </c>
-      <c r="I17" s="15" t="inlineStr">
-        <is>
-          <t>512-BC33740BU</t>
-        </is>
-      </c>
+          <t>870235673001</t>
+        </is>
+      </c>
+      <c r="I17" s="15" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="15" t="inlineStr">
         <is>
-          <t>R15</t>
+          <t>R13</t>
         </is>
       </c>
       <c r="B18" s="15" t="inlineStr">
         <is>
-          <t>220</t>
+          <t>220Ω</t>
         </is>
       </c>
       <c r="C18" s="15" t="inlineStr">
         <is>
-          <t>THT</t>
+          <t>SMD</t>
         </is>
       </c>
       <c r="D18" s="15" t="inlineStr">
@@ -5867,34 +5557,34 @@
       </c>
       <c r="F18" s="15" t="inlineStr">
         <is>
-          <t>Resistor_THT:R_Axial_DIN0617_L17.0mm_D6.0mm_P20.32mm_Horizontal</t>
+          <t>Resistor_SMD:R_0805_2012Metric</t>
         </is>
       </c>
       <c r="G18" s="15" t="inlineStr">
         <is>
-          <t>Vishay BC Components</t>
+          <t>YAGEO</t>
         </is>
       </c>
       <c r="H18" s="15" t="inlineStr">
         <is>
-          <t>PR02000202200JR500</t>
+          <t>RC0805FR-07220RL</t>
         </is>
       </c>
       <c r="I18" s="15" t="inlineStr">
         <is>
-          <t>594-5083NW220R0J</t>
+          <t>603-RC0805FR-07220RL</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="15" t="inlineStr">
         <is>
-          <t>C8</t>
+          <t>R9</t>
         </is>
       </c>
       <c r="B19" s="15" t="inlineStr">
         <is>
-          <t>WCAP-PT5H_6.3X5.2</t>
+          <t>10kΩ</t>
         </is>
       </c>
       <c r="C19" s="15" t="inlineStr">
@@ -5909,40 +5599,44 @@
       </c>
       <c r="E19" s="15" t="inlineStr">
         <is>
-          <t>WCAP-PT5H_6.3X5.2:WCAP-PT5H_6.3X5.2</t>
+          <t>Device:R</t>
         </is>
       </c>
       <c r="F19" s="15" t="inlineStr">
         <is>
-          <t>WCAP-PT5H_6.3X5.2:WCAP-PT5H_6.3X5.2_DXL_</t>
+          <t>Resistor_SMD:R_0805_2012Metric</t>
         </is>
       </c>
       <c r="G19" s="15" t="inlineStr">
         <is>
-          <t>Wurth Elektronik</t>
+          <t>YAGEO</t>
         </is>
       </c>
       <c r="H19" s="15" t="inlineStr">
         <is>
-          <t>870235673001</t>
-        </is>
-      </c>
-      <c r="I19" s="15" t="inlineStr"/>
+          <t>RC0805FR-0710KL</t>
+        </is>
+      </c>
+      <c r="I19" s="15" t="inlineStr">
+        <is>
+          <t>603-RC0805FR-0710KL</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="15" t="inlineStr">
         <is>
-          <t>R13</t>
+          <t>D8</t>
         </is>
       </c>
       <c r="B20" s="15" t="inlineStr">
         <is>
-          <t>220</t>
+          <t>BLUE</t>
         </is>
       </c>
       <c r="C20" s="15" t="inlineStr">
         <is>
-          <t>THT</t>
+          <t>SMD</t>
         </is>
       </c>
       <c r="D20" s="15" t="inlineStr">
@@ -5952,44 +5646,44 @@
       </c>
       <c r="E20" s="15" t="inlineStr">
         <is>
-          <t>Device:R</t>
+          <t>Device:LED</t>
         </is>
       </c>
       <c r="F20" s="15" t="inlineStr">
         <is>
-          <t>Resistor_THT:R_Axial_DIN0617_L17.0mm_D6.0mm_P20.32mm_Horizontal</t>
+          <t>LED_THT:LED_D3.0mm_Horizontal_O1.27mm_Z2.0mm</t>
         </is>
       </c>
       <c r="G20" s="15" t="inlineStr">
         <is>
-          <t>Vishay BC Components</t>
+          <t>Würth Elektronik</t>
         </is>
       </c>
       <c r="H20" s="15" t="inlineStr">
         <is>
-          <t>PR02000202200JR500</t>
+          <t>151033BS03000</t>
         </is>
       </c>
       <c r="I20" s="15" t="inlineStr">
         <is>
-          <t>594-5083NW220R0J</t>
+          <t>710-151033BS03000</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="15" t="inlineStr">
         <is>
-          <t>R26</t>
+          <t>C7</t>
         </is>
       </c>
       <c r="B21" s="15" t="inlineStr">
         <is>
-          <t>4,7k</t>
+          <t>WCAP-FTXX_P10</t>
         </is>
       </c>
       <c r="C21" s="15" t="inlineStr">
         <is>
-          <t>THT</t>
+          <t>SMD</t>
         </is>
       </c>
       <c r="D21" s="15" t="inlineStr">
@@ -5999,44 +5693,40 @@
       </c>
       <c r="E21" s="15" t="inlineStr">
         <is>
-          <t>Device:R</t>
+          <t>WCAP-FTXX_P10:WCAP-FTXX_P10</t>
         </is>
       </c>
       <c r="F21" s="15" t="inlineStr">
         <is>
-          <t>Resistor_THT:R_Axial_DIN0617_L17.0mm_D6.0mm_P20.32mm_Horizontal</t>
+          <t>WCAP-FTXX_P10:WCAP-FTXX_P10L13W7H13</t>
         </is>
       </c>
       <c r="G21" s="15" t="inlineStr">
         <is>
-          <t>Vishay BC Components</t>
+          <t>Würth Elektronik</t>
         </is>
       </c>
       <c r="H21" s="15" t="inlineStr">
         <is>
-          <t>PR02000204701JR500</t>
-        </is>
-      </c>
-      <c r="I21" s="15" t="inlineStr">
-        <is>
-          <t>594-5083NW4K700J</t>
-        </is>
-      </c>
+          <t>890334023023</t>
+        </is>
+      </c>
+      <c r="I21" s="15" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="15" t="inlineStr">
         <is>
-          <t>R9</t>
+          <t>D10</t>
         </is>
       </c>
       <c r="B22" s="15" t="inlineStr">
         <is>
-          <t>10k</t>
+          <t>GREEN</t>
         </is>
       </c>
       <c r="C22" s="15" t="inlineStr">
         <is>
-          <t>THT</t>
+          <t>SMD</t>
         </is>
       </c>
       <c r="D22" s="15" t="inlineStr">
@@ -6046,39 +5736,39 @@
       </c>
       <c r="E22" s="15" t="inlineStr">
         <is>
-          <t>Device:R</t>
+          <t>Device:LED</t>
         </is>
       </c>
       <c r="F22" s="15" t="inlineStr">
         <is>
-          <t>Resistor_THT:R_Axial_DIN0207_L6.3mm_D2.5mm_P10.16mm_Horizontal</t>
+          <t>LED_THT:LED_D3.0mm_Horizontal_O1.27mm_Z2.0mm</t>
         </is>
       </c>
       <c r="G22" s="15" t="inlineStr">
         <is>
-          <t>YAGEO</t>
+          <t>Würth Elektronik</t>
         </is>
       </c>
       <c r="H22" s="15" t="inlineStr">
         <is>
-          <t>MFR-25FBF52-10K</t>
+          <t>151031VS06000</t>
         </is>
       </c>
       <c r="I22" s="15" t="inlineStr">
         <is>
-          <t>603-MFR-25FBF52-10K</t>
+          <t>710-151031VS06000</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="15" t="inlineStr">
         <is>
-          <t>R23</t>
+          <t>S2</t>
         </is>
       </c>
       <c r="B23" s="15" t="inlineStr">
         <is>
-          <t>4,7k</t>
+          <t>PTS645VL58-2 LFS</t>
         </is>
       </c>
       <c r="C23" s="15" t="inlineStr">
@@ -6093,44 +5783,44 @@
       </c>
       <c r="E23" s="15" t="inlineStr">
         <is>
-          <t>Device:R</t>
+          <t>1543-650-149:1543-650-149</t>
         </is>
       </c>
       <c r="F23" s="15" t="inlineStr">
         <is>
-          <t>Resistor_THT:R_Axial_DIN0617_L17.0mm_D6.0mm_P20.32mm_Horizontal</t>
+          <t>PTS645VL58-2LFS:SW_Tactile_SPST_Angled_PTS645Vx58-2LFS</t>
         </is>
       </c>
       <c r="G23" s="15" t="inlineStr">
         <is>
-          <t>Vishay BC Components</t>
+          <t>C&amp;K</t>
         </is>
       </c>
       <c r="H23" s="15" t="inlineStr">
         <is>
-          <t>PR02000204701JR500</t>
+          <t>PTS645VL58-2 LFS</t>
         </is>
       </c>
       <c r="I23" s="15" t="inlineStr">
         <is>
-          <t>594-5083NW4K700J</t>
+          <t>611-PTS645VL582</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="15" t="inlineStr">
         <is>
-          <t>D8</t>
+          <t>U6</t>
         </is>
       </c>
       <c r="B24" s="15" t="inlineStr">
         <is>
-          <t>BLUE</t>
+          <t>ESP32-S3-WROOM-1U-N16R8</t>
         </is>
       </c>
       <c r="C24" s="15" t="inlineStr">
         <is>
-          <t>THT</t>
+          <t>SMD</t>
         </is>
       </c>
       <c r="D24" s="15" t="inlineStr">
@@ -6140,34 +5830,34 @@
       </c>
       <c r="E24" s="15" t="inlineStr">
         <is>
-          <t>Device:LED</t>
+          <t>ESP32-S3-WROOM-1U-N16R8:ESP32-S3-WROOM-1U-N16R8</t>
         </is>
       </c>
       <c r="F24" s="15" t="inlineStr">
         <is>
-          <t>WL-TMRW_3MM:WL-TMRW_3MM</t>
+          <t>ESP32-S3-WROOM-1U-N16R8:ESP32-S3-WROOM-1U</t>
         </is>
       </c>
       <c r="G24" s="15" t="inlineStr">
         <is>
-          <t>Würth Elektronik</t>
+          <t>Espressif Systems</t>
         </is>
       </c>
       <c r="H24" s="15" t="inlineStr">
         <is>
-          <t>151033BS03000</t>
+          <t>ESP32-S3-WROOM-1U-N16R8</t>
         </is>
       </c>
       <c r="I24" s="15" t="inlineStr">
         <is>
-          <t>710-151033BS03000</t>
+          <t>356-ESP32S3WM1UN16R8</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="15" t="inlineStr">
         <is>
-          <t>C7</t>
+          <t>C12</t>
         </is>
       </c>
       <c r="B25" s="15" t="inlineStr">
@@ -6210,12 +5900,12 @@
     <row r="26">
       <c r="A26" s="15" t="inlineStr">
         <is>
-          <t>D10</t>
+          <t>J6</t>
         </is>
       </c>
       <c r="B26" s="15" t="inlineStr">
         <is>
-          <t>GREEN</t>
+          <t>61200621621</t>
         </is>
       </c>
       <c r="C26" s="15" t="inlineStr">
@@ -6230,12 +5920,12 @@
       </c>
       <c r="E26" s="15" t="inlineStr">
         <is>
-          <t>Device:LED</t>
+          <t>Connector_Generic:Conn_02x03_Odd_Even</t>
         </is>
       </c>
       <c r="F26" s="15" t="inlineStr">
         <is>
-          <t>WL-TMRC_3MM:WL-TMRC_3MM</t>
+          <t>wuerth_6120XX21621:61200621621</t>
         </is>
       </c>
       <c r="G26" s="15" t="inlineStr">
@@ -6245,29 +5935,29 @@
       </c>
       <c r="H26" s="15" t="inlineStr">
         <is>
-          <t>151031VS06000</t>
+          <t>61200621621</t>
         </is>
       </c>
       <c r="I26" s="15" t="inlineStr">
         <is>
-          <t>710-151031VS06000</t>
+          <t>710-61200621621</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="15" t="inlineStr">
         <is>
-          <t>Q3</t>
+          <t>R16</t>
         </is>
       </c>
       <c r="B27" s="15" t="inlineStr">
         <is>
-          <t>BC337</t>
+          <t>220Ω</t>
         </is>
       </c>
       <c r="C27" s="15" t="inlineStr">
         <is>
-          <t>THT</t>
+          <t>SMD</t>
         </is>
       </c>
       <c r="D27" s="15" t="inlineStr">
@@ -6277,180 +5967,180 @@
       </c>
       <c r="E27" s="15" t="inlineStr">
         <is>
-          <t>Transistor_BJT:BC337</t>
+          <t>Device:R</t>
         </is>
       </c>
       <c r="F27" s="15" t="inlineStr">
         <is>
-          <t>Package_TO_SOT_THT:TO-92_Inline</t>
+          <t>Resistor_SMD:R_0805_2012Metric</t>
         </is>
       </c>
       <c r="G27" s="15" t="inlineStr">
         <is>
-          <t>onsemi</t>
+          <t>YAGEO</t>
         </is>
       </c>
       <c r="H27" s="15" t="inlineStr">
         <is>
-          <t>BC33740BU</t>
+          <t>RC0805FR-07220RL</t>
         </is>
       </c>
       <c r="I27" s="15" t="inlineStr">
         <is>
-          <t>512-BC33740BU</t>
+          <t>603-RC0805FR-07220RL</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="15" t="inlineStr">
         <is>
-          <t>S2</t>
+          <t>R20</t>
         </is>
       </c>
       <c r="B28" s="15" t="inlineStr">
         <is>
-          <t>PTS645VL58-2 LFS</t>
+          <t>5,1 kΩ</t>
         </is>
       </c>
       <c r="C28" s="15" t="inlineStr">
         <is>
-          <t>THT</t>
+          <t>SMD</t>
         </is>
       </c>
       <c r="D28" s="15" t="inlineStr">
         <is>
-          <t>BasisStation_Layout.kicad_sch</t>
+          <t>Stromversorgung.kicad_sch</t>
         </is>
       </c>
       <c r="E28" s="15" t="inlineStr">
         <is>
-          <t>1543-650-149:1543-650-149</t>
+          <t>Device:R</t>
         </is>
       </c>
       <c r="F28" s="15" t="inlineStr">
         <is>
-          <t>PTS645VL58-2LFS:SW_Tactile_SPST_Angled_PTS645Vx58-2LFS</t>
+          <t>Resistor_SMD:R_0805_2012Metric</t>
         </is>
       </c>
       <c r="G28" s="15" t="inlineStr">
         <is>
-          <t>C&amp;K</t>
+          <t>YAGEO</t>
         </is>
       </c>
       <c r="H28" s="15" t="inlineStr">
         <is>
-          <t>PTS645VL58-2 LFS</t>
+          <t>RC0805FR-075K1L</t>
         </is>
       </c>
       <c r="I28" s="15" t="inlineStr">
         <is>
-          <t>611-PTS645VL582</t>
+          <t>603-RC0805FR-075K1L</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="15" t="inlineStr">
         <is>
-          <t>U6</t>
+          <t>J_PWR1</t>
         </is>
       </c>
       <c r="B29" s="15" t="inlineStr">
         <is>
-          <t>ESP32-S3-WROOM-1U-N16R8</t>
+          <t>12401598E4-2A</t>
         </is>
       </c>
       <c r="C29" s="15" t="inlineStr">
         <is>
-          <t>SMD</t>
+          <t>THT</t>
         </is>
       </c>
       <c r="D29" s="15" t="inlineStr">
         <is>
-          <t>BasisStation_Layout.kicad_sch</t>
+          <t>Stromversorgung.kicad_sch</t>
         </is>
       </c>
       <c r="E29" s="15" t="inlineStr">
         <is>
-          <t>ESP32-S3-WROOM-1U-N16R8:ESP32-S3-WROOM-1U-N16R8</t>
+          <t>shbs_power:USB_C_Receptacle_Power</t>
         </is>
       </c>
       <c r="F29" s="15" t="inlineStr">
         <is>
-          <t>ESP32-S3-WROOM-1U-N16R8:ESP32-S3-WROOM-1U</t>
+          <t>shbs_power:USB_C_Receptacle_Amphenol_12401598E4-2A</t>
         </is>
       </c>
       <c r="G29" s="15" t="inlineStr">
         <is>
-          <t>Espressif Systems</t>
+          <t>Amphenol</t>
         </is>
       </c>
       <c r="H29" s="15" t="inlineStr">
         <is>
-          <t>ESP32-S3-WROOM-1U-N16R8</t>
+          <t>12401598E4#2A</t>
         </is>
       </c>
       <c r="I29" s="15" t="inlineStr">
         <is>
-          <t>356-ESP32S3WM1UN16R8</t>
+          <t>523-12401598E4#2A</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="15" t="inlineStr">
         <is>
-          <t>R24</t>
+          <t>C13</t>
         </is>
       </c>
       <c r="B30" s="15" t="inlineStr">
         <is>
-          <t>4,7k</t>
+          <t>10uF</t>
         </is>
       </c>
       <c r="C30" s="15" t="inlineStr">
         <is>
-          <t>THT</t>
+          <t>SMD</t>
         </is>
       </c>
       <c r="D30" s="15" t="inlineStr">
         <is>
-          <t>BasisStation_Layout.kicad_sch</t>
+          <t>Stromversorgung.kicad_sch</t>
         </is>
       </c>
       <c r="E30" s="15" t="inlineStr">
         <is>
-          <t>Device:R</t>
+          <t>Device:C</t>
         </is>
       </c>
       <c r="F30" s="15" t="inlineStr">
         <is>
-          <t>Resistor_THT:R_Axial_DIN0617_L17.0mm_D6.0mm_P20.32mm_Horizontal</t>
+          <t>Capacitor_SMD:C_0805_2012Metric</t>
         </is>
       </c>
       <c r="G30" s="15" t="inlineStr">
         <is>
-          <t>Vishay BC Components</t>
+          <t>Samsung</t>
         </is>
       </c>
       <c r="H30" s="15" t="inlineStr">
         <is>
-          <t>PR02000204701JR500</t>
+          <t>CL21B106KOQNNNE</t>
         </is>
       </c>
       <c r="I30" s="15" t="inlineStr">
         <is>
-          <t>594-5083NW4K700J</t>
+          <t>187-CL21B106KOQNNNE</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="15" t="inlineStr">
         <is>
-          <t>C12</t>
+          <t>D11</t>
         </is>
       </c>
       <c r="B31" s="15" t="inlineStr">
         <is>
-          <t>WCAP-FTXX_P10</t>
+          <t>SS34</t>
         </is>
       </c>
       <c r="C31" s="15" t="inlineStr">
@@ -6460,97 +6150,101 @@
       </c>
       <c r="D31" s="15" t="inlineStr">
         <is>
-          <t>BasisStation_Layout.kicad_sch</t>
+          <t>Stromversorgung.kicad_sch</t>
         </is>
       </c>
       <c r="E31" s="15" t="inlineStr">
         <is>
-          <t>WCAP-FTXX_P10:WCAP-FTXX_P10</t>
+          <t>Diode:SS34</t>
         </is>
       </c>
       <c r="F31" s="15" t="inlineStr">
         <is>
-          <t>WCAP-FTXX_P10:WCAP-FTXX_P10L13W7H13</t>
+          <t>Diode_SMD:D_SMA</t>
         </is>
       </c>
       <c r="G31" s="15" t="inlineStr">
         <is>
-          <t>Würth Elektronik</t>
+          <t>Comchip Technology</t>
         </is>
       </c>
       <c r="H31" s="15" t="inlineStr">
         <is>
-          <t>890334023023</t>
-        </is>
-      </c>
-      <c r="I31" s="15" t="inlineStr"/>
+          <t>SS34-HF</t>
+        </is>
+      </c>
+      <c r="I31" s="15" t="inlineStr">
+        <is>
+          <t>750-SS34-HF</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="15" t="inlineStr">
         <is>
-          <t>J6</t>
+          <t>F1</t>
         </is>
       </c>
       <c r="B32" s="15" t="inlineStr">
         <is>
-          <t>61200621621</t>
+          <t>1.1A</t>
         </is>
       </c>
       <c r="C32" s="15" t="inlineStr">
         <is>
-          <t>THT</t>
+          <t>SMD</t>
         </is>
       </c>
       <c r="D32" s="15" t="inlineStr">
         <is>
-          <t>BasisStation_Layout.kicad_sch</t>
+          <t>Stromversorgung.kicad_sch</t>
         </is>
       </c>
       <c r="E32" s="15" t="inlineStr">
         <is>
-          <t>Connector_Generic:Conn_02x03_Odd_Even</t>
+          <t>Device:Fuse</t>
         </is>
       </c>
       <c r="F32" s="15" t="inlineStr">
         <is>
-          <t>wuerth_6120XX21621:61200621621</t>
+          <t>Fuse:Fuse_1206_3216Metric</t>
         </is>
       </c>
       <c r="G32" s="15" t="inlineStr">
         <is>
-          <t>Würth Elektronik</t>
+          <t>Bourns</t>
         </is>
       </c>
       <c r="H32" s="15" t="inlineStr">
         <is>
-          <t>61200621621</t>
+          <t>MF-NSMF110-2</t>
         </is>
       </c>
       <c r="I32" s="15" t="inlineStr">
         <is>
-          <t>710-61200621621</t>
+          <t>652-MF-NSMF110-2</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="15" t="inlineStr">
         <is>
-          <t>R25</t>
+          <t>R18</t>
         </is>
       </c>
       <c r="B33" s="15" t="inlineStr">
         <is>
-          <t>4,7k</t>
+          <t>16,2 kΩ</t>
         </is>
       </c>
       <c r="C33" s="15" t="inlineStr">
         <is>
-          <t>THT</t>
+          <t>SMD</t>
         </is>
       </c>
       <c r="D33" s="15" t="inlineStr">
         <is>
-          <t>BasisStation_Layout.kicad_sch</t>
+          <t>Stromversorgung.kicad_sch</t>
         </is>
       </c>
       <c r="E33" s="15" t="inlineStr">
@@ -6560,128 +6254,128 @@
       </c>
       <c r="F33" s="15" t="inlineStr">
         <is>
-          <t>Resistor_THT:R_Axial_DIN0617_L17.0mm_D6.0mm_P20.32mm_Horizontal</t>
+          <t>Resistor_SMD:R_0805_2012Metric</t>
         </is>
       </c>
       <c r="G33" s="15" t="inlineStr">
         <is>
-          <t>Vishay BC Components</t>
+          <t>YAGEO</t>
         </is>
       </c>
       <c r="H33" s="15" t="inlineStr">
         <is>
-          <t>PR02000204701JR500</t>
+          <t>RC0805FR-0716K2L</t>
         </is>
       </c>
       <c r="I33" s="15" t="inlineStr">
         <is>
-          <t>594-5083NW4K700J</t>
+          <t>603-RC0805FR-0716K2L</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="15" t="inlineStr">
         <is>
-          <t>Q2</t>
+          <t>C14</t>
         </is>
       </c>
       <c r="B34" s="15" t="inlineStr">
         <is>
-          <t>BC337</t>
+          <t>22uF</t>
         </is>
       </c>
       <c r="C34" s="15" t="inlineStr">
         <is>
-          <t>THT</t>
+          <t>SMD</t>
         </is>
       </c>
       <c r="D34" s="15" t="inlineStr">
         <is>
-          <t>BasisStation_Layout.kicad_sch</t>
+          <t>Stromversorgung.kicad_sch</t>
         </is>
       </c>
       <c r="E34" s="15" t="inlineStr">
         <is>
-          <t>Transistor_BJT:BC337</t>
+          <t>Device:C</t>
         </is>
       </c>
       <c r="F34" s="15" t="inlineStr">
         <is>
-          <t>Package_TO_SOT_THT:TO-92_Inline</t>
+          <t>Capacitor_SMD:C_0805_2012Metric</t>
         </is>
       </c>
       <c r="G34" s="15" t="inlineStr">
         <is>
-          <t>onsemi</t>
+          <t>Samsung</t>
         </is>
       </c>
       <c r="H34" s="15" t="inlineStr">
         <is>
-          <t>BC33740BU</t>
+          <t>CL21A226MOQNNNE</t>
         </is>
       </c>
       <c r="I34" s="15" t="inlineStr">
         <is>
-          <t>512-BC33740BU</t>
+          <t>187-CL21A226MOQNNNE</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="15" t="inlineStr">
         <is>
-          <t>R16</t>
+          <t>C15</t>
         </is>
       </c>
       <c r="B35" s="15" t="inlineStr">
         <is>
-          <t>220</t>
+          <t>100 nF</t>
         </is>
       </c>
       <c r="C35" s="15" t="inlineStr">
         <is>
-          <t>THT</t>
+          <t>SMD</t>
         </is>
       </c>
       <c r="D35" s="15" t="inlineStr">
         <is>
-          <t>BasisStation_Layout.kicad_sch</t>
+          <t>Stromversorgung.kicad_sch</t>
         </is>
       </c>
       <c r="E35" s="15" t="inlineStr">
         <is>
-          <t>Device:R</t>
+          <t>Device:C</t>
         </is>
       </c>
       <c r="F35" s="15" t="inlineStr">
         <is>
-          <t>Resistor_THT:R_Axial_DIN0617_L17.0mm_D6.0mm_P20.32mm_Horizontal</t>
+          <t>Capacitor_SMD:C_0805_2012Metric</t>
         </is>
       </c>
       <c r="G35" s="15" t="inlineStr">
         <is>
-          <t>Vishay BC Components</t>
+          <t>YAGEO</t>
         </is>
       </c>
       <c r="H35" s="15" t="inlineStr">
         <is>
-          <t>PR02000202200JR500</t>
+          <t>CC0805KRX7R9BB104</t>
         </is>
       </c>
       <c r="I35" s="15" t="inlineStr">
         <is>
-          <t>594-5083NW220R0J</t>
+          <t>603-CC805KRX7R9BB104</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="15" t="inlineStr">
         <is>
-          <t>R20</t>
+          <t>D12</t>
         </is>
       </c>
       <c r="B36" s="15" t="inlineStr">
         <is>
-          <t>5,1 kΩ</t>
+          <t>SMAJ5.0A</t>
         </is>
       </c>
       <c r="C36" s="15" t="inlineStr">
@@ -6696,44 +6390,44 @@
       </c>
       <c r="E36" s="15" t="inlineStr">
         <is>
-          <t>Device:R</t>
+          <t>Diode:SMAJ5.0A</t>
         </is>
       </c>
       <c r="F36" s="15" t="inlineStr">
         <is>
-          <t>Resistor_SMD:R_0805_2012Metric</t>
+          <t>Diode_SMD:D_SMA</t>
         </is>
       </c>
       <c r="G36" s="15" t="inlineStr">
         <is>
-          <t>YAGEO</t>
+          <t>Littelfuse</t>
         </is>
       </c>
       <c r="H36" s="15" t="inlineStr">
         <is>
-          <t>RC0805FR-075K1L</t>
+          <t>SMAJ5.0A</t>
         </is>
       </c>
       <c r="I36" s="15" t="inlineStr">
         <is>
-          <t>603-RC0805FR-075K1L</t>
+          <t>576-SMAJ5.0A</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="15" t="inlineStr">
         <is>
-          <t>J_PWR1</t>
+          <t>PS1</t>
         </is>
       </c>
       <c r="B37" s="15" t="inlineStr">
         <is>
-          <t>12401598E4-2A</t>
+          <t>AP3211</t>
         </is>
       </c>
       <c r="C37" s="15" t="inlineStr">
         <is>
-          <t>THT</t>
+          <t>SMD</t>
         </is>
       </c>
       <c r="D37" s="15" t="inlineStr">
@@ -6743,39 +6437,39 @@
       </c>
       <c r="E37" s="15" t="inlineStr">
         <is>
-          <t>shbs_power:USB_C_Receptacle_Power</t>
+          <t>shbs_power:AP3211</t>
         </is>
       </c>
       <c r="F37" s="15" t="inlineStr">
         <is>
-          <t>shbs_power:USB_C_Receptacle_Amphenol_12401598E4-2A</t>
+          <t>shbs_power:MP2359DJ</t>
         </is>
       </c>
       <c r="G37" s="15" t="inlineStr">
         <is>
-          <t>Amphenol</t>
+          <t>Diodes Incorporated</t>
         </is>
       </c>
       <c r="H37" s="15" t="inlineStr">
         <is>
-          <t>12401598E4#2A</t>
+          <t>AP3211KTR-G1</t>
         </is>
       </c>
       <c r="I37" s="15" t="inlineStr">
         <is>
-          <t>523-12401598E4#2A</t>
+          <t>621-AP3211KTR-G1</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="15" t="inlineStr">
         <is>
-          <t>C13</t>
+          <t>R17</t>
         </is>
       </c>
       <c r="B38" s="15" t="inlineStr">
         <is>
-          <t>10uF</t>
+          <t>49,9 kΩ</t>
         </is>
       </c>
       <c r="C38" s="15" t="inlineStr">
@@ -6790,39 +6484,39 @@
       </c>
       <c r="E38" s="15" t="inlineStr">
         <is>
-          <t>Device:C</t>
+          <t>Device:R</t>
         </is>
       </c>
       <c r="F38" s="15" t="inlineStr">
         <is>
-          <t>Capacitor_SMD:C_0805_2012Metric</t>
+          <t>Resistor_SMD:R_0805_2012Metric</t>
         </is>
       </c>
       <c r="G38" s="15" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>YAGEO</t>
         </is>
       </c>
       <c r="H38" s="15" t="inlineStr">
         <is>
-          <t>CL21B106KOQNNNE</t>
+          <t>RC0805FR-0749K9L</t>
         </is>
       </c>
       <c r="I38" s="15" t="inlineStr">
         <is>
-          <t>187-CL21B106KOQNNNE</t>
+          <t>603-RC0805FR-0749K9L</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="15" t="inlineStr">
         <is>
-          <t>D11</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="B39" s="15" t="inlineStr">
         <is>
-          <t>SS34</t>
+          <t>10uH</t>
         </is>
       </c>
       <c r="C39" s="15" t="inlineStr">
@@ -6837,39 +6531,39 @@
       </c>
       <c r="E39" s="15" t="inlineStr">
         <is>
-          <t>Diode:SS34</t>
+          <t>Device:L</t>
         </is>
       </c>
       <c r="F39" s="15" t="inlineStr">
         <is>
-          <t>Diode_SMD:D_SMA</t>
+          <t>Inductor_SMD:L_Bourns_SRN6045TA</t>
         </is>
       </c>
       <c r="G39" s="15" t="inlineStr">
         <is>
-          <t>Comchip Technology</t>
+          <t>Bourns</t>
         </is>
       </c>
       <c r="H39" s="15" t="inlineStr">
         <is>
-          <t>SS34-HF</t>
+          <t>SRN6045TA-100M</t>
         </is>
       </c>
       <c r="I39" s="15" t="inlineStr">
         <is>
-          <t>750-SS34-HF</t>
+          <t>652-SRN6045TA-100M</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="15" t="inlineStr">
         <is>
-          <t>F1</t>
+          <t>R19</t>
         </is>
       </c>
       <c r="B40" s="15" t="inlineStr">
         <is>
-          <t>1.1A</t>
+          <t>5,1 kΩ</t>
         </is>
       </c>
       <c r="C40" s="15" t="inlineStr">
@@ -6884,39 +6578,39 @@
       </c>
       <c r="E40" s="15" t="inlineStr">
         <is>
-          <t>Device:Fuse</t>
+          <t>Device:R</t>
         </is>
       </c>
       <c r="F40" s="15" t="inlineStr">
         <is>
-          <t>Fuse:Fuse_1206_3216Metric</t>
+          <t>Resistor_SMD:R_0805_2012Metric</t>
         </is>
       </c>
       <c r="G40" s="15" t="inlineStr">
         <is>
-          <t>Bourns</t>
+          <t>YAGEO</t>
         </is>
       </c>
       <c r="H40" s="15" t="inlineStr">
         <is>
-          <t>MF-NSMF110-2</t>
+          <t>RC0805FR-075K1L</t>
         </is>
       </c>
       <c r="I40" s="15" t="inlineStr">
         <is>
-          <t>652-MF-NSMF110-2</t>
+          <t>603-RC0805FR-075K1L</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="15" t="inlineStr">
         <is>
-          <t>R18</t>
+          <t>R33</t>
         </is>
       </c>
       <c r="B41" s="15" t="inlineStr">
         <is>
-          <t>16,2 kΩ</t>
+          <t>220Ω</t>
         </is>
       </c>
       <c r="C41" s="15" t="inlineStr">
@@ -6926,7 +6620,7 @@
       </c>
       <c r="D41" s="15" t="inlineStr">
         <is>
-          <t>Stromversorgung.kicad_sch</t>
+          <t>ethernet.kicad_sch</t>
         </is>
       </c>
       <c r="E41" s="15" t="inlineStr">
@@ -6946,24 +6640,24 @@
       </c>
       <c r="H41" s="15" t="inlineStr">
         <is>
-          <t>RC0805FR-0716K2L</t>
+          <t>RC0805FR-07220RL</t>
         </is>
       </c>
       <c r="I41" s="15" t="inlineStr">
         <is>
-          <t>603-RC0805FR-0716K2L</t>
+          <t>603-RC0805FR-07220RL</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="15" t="inlineStr">
         <is>
-          <t>C14</t>
+          <t>R34</t>
         </is>
       </c>
       <c r="B42" s="15" t="inlineStr">
         <is>
-          <t>22uF</t>
+          <t>220Ω</t>
         </is>
       </c>
       <c r="C42" s="15" t="inlineStr">
@@ -6973,44 +6667,44 @@
       </c>
       <c r="D42" s="15" t="inlineStr">
         <is>
-          <t>Stromversorgung.kicad_sch</t>
+          <t>ethernet.kicad_sch</t>
         </is>
       </c>
       <c r="E42" s="15" t="inlineStr">
         <is>
-          <t>Device:C</t>
+          <t>Device:R</t>
         </is>
       </c>
       <c r="F42" s="15" t="inlineStr">
         <is>
-          <t>Capacitor_SMD:C_0805_2012Metric</t>
+          <t>Resistor_SMD:R_0805_2012Metric</t>
         </is>
       </c>
       <c r="G42" s="15" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>YAGEO</t>
         </is>
       </c>
       <c r="H42" s="15" t="inlineStr">
         <is>
-          <t>CL21A226MOQNNNE</t>
+          <t>RC0805FR-07220RL</t>
         </is>
       </c>
       <c r="I42" s="15" t="inlineStr">
         <is>
-          <t>187-CL21A226MOQNNNE</t>
+          <t>603-RC0805FR-07220RL</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="15" t="inlineStr">
         <is>
-          <t>C15</t>
+          <t>C16</t>
         </is>
       </c>
       <c r="B43" s="15" t="inlineStr">
         <is>
-          <t>100 nF</t>
+          <t>100nF</t>
         </is>
       </c>
       <c r="C43" s="15" t="inlineStr">
@@ -7020,7 +6714,7 @@
       </c>
       <c r="D43" s="15" t="inlineStr">
         <is>
-          <t>Stromversorgung.kicad_sch</t>
+          <t>ethernet.kicad_sch</t>
         </is>
       </c>
       <c r="E43" s="15" t="inlineStr">
@@ -7052,12 +6746,12 @@
     <row r="44">
       <c r="A44" s="15" t="inlineStr">
         <is>
-          <t>D12</t>
+          <t>FB1</t>
         </is>
       </c>
       <c r="B44" s="15" t="inlineStr">
         <is>
-          <t>SMAJ5.0A</t>
+          <t>Ferrit 600R@100MHz</t>
         </is>
       </c>
       <c r="C44" s="15" t="inlineStr">
@@ -7067,44 +6761,44 @@
       </c>
       <c r="D44" s="15" t="inlineStr">
         <is>
-          <t>Stromversorgung.kicad_sch</t>
+          <t>ethernet.kicad_sch</t>
         </is>
       </c>
       <c r="E44" s="15" t="inlineStr">
         <is>
-          <t>Diode:SMAJ5.0A</t>
+          <t>Device:FerriteBead</t>
         </is>
       </c>
       <c r="F44" s="15" t="inlineStr">
         <is>
-          <t>Diode_SMD:D_SMA</t>
+          <t>Inductor_SMD:L_0805_2012Metric</t>
         </is>
       </c>
       <c r="G44" s="15" t="inlineStr">
         <is>
-          <t>Littelfuse</t>
+          <t>Murata</t>
         </is>
       </c>
       <c r="H44" s="15" t="inlineStr">
         <is>
-          <t>SMAJ5.0A</t>
+          <t>BLM21PG601SN1D</t>
         </is>
       </c>
       <c r="I44" s="15" t="inlineStr">
         <is>
-          <t>576-SMAJ5.0A</t>
+          <t>81-BLM21PG601SN1D</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="15" t="inlineStr">
         <is>
-          <t>PS1</t>
+          <t>U7</t>
         </is>
       </c>
       <c r="B45" s="15" t="inlineStr">
         <is>
-          <t>AP3211</t>
+          <t>W5500</t>
         </is>
       </c>
       <c r="C45" s="15" t="inlineStr">
@@ -7114,44 +6808,40 @@
       </c>
       <c r="D45" s="15" t="inlineStr">
         <is>
-          <t>Stromversorgung.kicad_sch</t>
+          <t>ethernet.kicad_sch</t>
         </is>
       </c>
       <c r="E45" s="15" t="inlineStr">
         <is>
-          <t>shbs_power:AP3211</t>
+          <t>W5500:W5500</t>
         </is>
       </c>
       <c r="F45" s="15" t="inlineStr">
         <is>
-          <t>shbs_power:MP2359DJ</t>
+          <t>W5500:48LQFP_W5500_WIZ</t>
         </is>
       </c>
       <c r="G45" s="15" t="inlineStr">
         <is>
-          <t>Diodes Incorporated</t>
+          <t>WIZnet</t>
         </is>
       </c>
       <c r="H45" s="15" t="inlineStr">
         <is>
-          <t>AP3211KTR-G1</t>
-        </is>
-      </c>
-      <c r="I45" s="15" t="inlineStr">
-        <is>
-          <t>621-AP3211KTR-G1</t>
-        </is>
-      </c>
+          <t>W5500</t>
+        </is>
+      </c>
+      <c r="I45" s="15" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="15" t="inlineStr">
         <is>
-          <t>R17</t>
+          <t>R35</t>
         </is>
       </c>
       <c r="B46" s="15" t="inlineStr">
         <is>
-          <t>49,9 kΩ</t>
+          <t>0Ω</t>
         </is>
       </c>
       <c r="C46" s="15" t="inlineStr">
@@ -7161,7 +6851,7 @@
       </c>
       <c r="D46" s="15" t="inlineStr">
         <is>
-          <t>Stromversorgung.kicad_sch</t>
+          <t>ethernet.kicad_sch</t>
         </is>
       </c>
       <c r="E46" s="15" t="inlineStr">
@@ -7181,24 +6871,24 @@
       </c>
       <c r="H46" s="15" t="inlineStr">
         <is>
-          <t>RC0805FR-0749K9L</t>
+          <t>RC0805JR-070RL</t>
         </is>
       </c>
       <c r="I46" s="15" t="inlineStr">
         <is>
-          <t>603-RC0805FR-0749K9L</t>
+          <t>603-RC0805JR-070RL</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="15" t="inlineStr">
         <is>
-          <t>L1</t>
+          <t>R39</t>
         </is>
       </c>
       <c r="B47" s="15" t="inlineStr">
         <is>
-          <t>10uH</t>
+          <t>49,9Ω 1%</t>
         </is>
       </c>
       <c r="C47" s="15" t="inlineStr">
@@ -7208,44 +6898,44 @@
       </c>
       <c r="D47" s="15" t="inlineStr">
         <is>
-          <t>Stromversorgung.kicad_sch</t>
+          <t>ethernet.kicad_sch</t>
         </is>
       </c>
       <c r="E47" s="15" t="inlineStr">
         <is>
-          <t>Device:L</t>
+          <t>Device:R</t>
         </is>
       </c>
       <c r="F47" s="15" t="inlineStr">
         <is>
-          <t>Inductor_SMD:L_Bourns_SRN6045TA</t>
+          <t>Resistor_SMD:R_0805_2012Metric</t>
         </is>
       </c>
       <c r="G47" s="15" t="inlineStr">
         <is>
-          <t>Bourns</t>
+          <t>YAGEO</t>
         </is>
       </c>
       <c r="H47" s="15" t="inlineStr">
         <is>
-          <t>SRN6045TA-100M</t>
+          <t>RC0805FR-0749R9L</t>
         </is>
       </c>
       <c r="I47" s="15" t="inlineStr">
         <is>
-          <t>652-SRN6045TA-100M</t>
+          <t>603-RC0805FR-0749R9L</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="15" t="inlineStr">
         <is>
-          <t>R19</t>
+          <t>Y1</t>
         </is>
       </c>
       <c r="B48" s="15" t="inlineStr">
         <is>
-          <t>5,1 kΩ</t>
+          <t>25 MHz</t>
         </is>
       </c>
       <c r="C48" s="15" t="inlineStr">
@@ -7255,44 +6945,44 @@
       </c>
       <c r="D48" s="15" t="inlineStr">
         <is>
-          <t>Stromversorgung.kicad_sch</t>
+          <t>ethernet.kicad_sch</t>
         </is>
       </c>
       <c r="E48" s="15" t="inlineStr">
         <is>
-          <t>Device:R</t>
+          <t>wuerth_xtal:CFPX-104_830059532</t>
         </is>
       </c>
       <c r="F48" s="15" t="inlineStr">
         <is>
-          <t>Resistor_SMD:R_0805_2012Metric</t>
+          <t>wuerth_830059532:Y_Wurth_WE-XTAL_Quartz-CFPX-104</t>
         </is>
       </c>
       <c r="G48" s="15" t="inlineStr">
         <is>
-          <t>YAGEO</t>
+          <t>Wurth Elektronik</t>
         </is>
       </c>
       <c r="H48" s="15" t="inlineStr">
         <is>
-          <t>RC0805FR-075K1L</t>
+          <t>830059532</t>
         </is>
       </c>
       <c r="I48" s="15" t="inlineStr">
         <is>
-          <t>603-RC0805FR-075K1L</t>
+          <t>710-830059532</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="15" t="inlineStr">
         <is>
-          <t>R33</t>
+          <t>C20</t>
         </is>
       </c>
       <c r="B49" s="15" t="inlineStr">
         <is>
-          <t>220Ω</t>
+          <t>100nF</t>
         </is>
       </c>
       <c r="C49" s="15" t="inlineStr">
@@ -7307,12 +6997,12 @@
       </c>
       <c r="E49" s="15" t="inlineStr">
         <is>
-          <t>Device:R</t>
+          <t>Device:C</t>
         </is>
       </c>
       <c r="F49" s="15" t="inlineStr">
         <is>
-          <t>Resistor_SMD:R_0805_2012Metric</t>
+          <t>Capacitor_SMD:C_0805_2012Metric</t>
         </is>
       </c>
       <c r="G49" s="15" t="inlineStr">
@@ -7322,24 +7012,24 @@
       </c>
       <c r="H49" s="15" t="inlineStr">
         <is>
-          <t>RC0805FR-07220RL</t>
+          <t>CC0805KRX7R9BB104</t>
         </is>
       </c>
       <c r="I49" s="15" t="inlineStr">
         <is>
-          <t>603-RC0805FR-07220RL</t>
+          <t>603-CC805KRX7R9BB104</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="15" t="inlineStr">
         <is>
-          <t>R34</t>
+          <t>R40</t>
         </is>
       </c>
       <c r="B50" s="15" t="inlineStr">
         <is>
-          <t>220Ω</t>
+          <t>49,9Ω 1%</t>
         </is>
       </c>
       <c r="C50" s="15" t="inlineStr">
@@ -7369,24 +7059,24 @@
       </c>
       <c r="H50" s="15" t="inlineStr">
         <is>
-          <t>RC0805FR-07220RL</t>
+          <t>RC0805FR-0749R9L</t>
         </is>
       </c>
       <c r="I50" s="15" t="inlineStr">
         <is>
-          <t>603-RC0805FR-07220RL</t>
+          <t>603-RC0805FR-0749R9L</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="15" t="inlineStr">
         <is>
-          <t>C16</t>
+          <t>R27</t>
         </is>
       </c>
       <c r="B51" s="15" t="inlineStr">
         <is>
-          <t>100nF</t>
+          <t>12,4kΩ, 1%</t>
         </is>
       </c>
       <c r="C51" s="15" t="inlineStr">
@@ -7401,12 +7091,12 @@
       </c>
       <c r="E51" s="15" t="inlineStr">
         <is>
-          <t>Device:C</t>
+          <t>Device:R</t>
         </is>
       </c>
       <c r="F51" s="15" t="inlineStr">
         <is>
-          <t>Capacitor_SMD:C_0805_2012Metric</t>
+          <t>Resistor_SMD:R_0805_2012Metric</t>
         </is>
       </c>
       <c r="G51" s="15" t="inlineStr">
@@ -7416,24 +7106,24 @@
       </c>
       <c r="H51" s="15" t="inlineStr">
         <is>
-          <t>CC0805KRX7R9BB104</t>
+          <t>RC0805FR-0712K4L</t>
         </is>
       </c>
       <c r="I51" s="15" t="inlineStr">
         <is>
-          <t>603-CC805KRX7R9BB104</t>
+          <t>603-RC0805FR-0712K4L</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="15" t="inlineStr">
         <is>
-          <t>FB1</t>
+          <t>R32</t>
         </is>
       </c>
       <c r="B52" s="15" t="inlineStr">
         <is>
-          <t>Ferrit 600R@100MHz</t>
+          <t>10kΩ</t>
         </is>
       </c>
       <c r="C52" s="15" t="inlineStr">
@@ -7448,39 +7138,39 @@
       </c>
       <c r="E52" s="15" t="inlineStr">
         <is>
-          <t>Device:FerriteBead</t>
+          <t>Device:R</t>
         </is>
       </c>
       <c r="F52" s="15" t="inlineStr">
         <is>
-          <t>Inductor_SMD:L_0805_2012Metric</t>
+          <t>Resistor_SMD:R_0805_2012Metric</t>
         </is>
       </c>
       <c r="G52" s="15" t="inlineStr">
         <is>
-          <t>Murata</t>
+          <t>YAGEO</t>
         </is>
       </c>
       <c r="H52" s="15" t="inlineStr">
         <is>
-          <t>BLM21PG601SN1D</t>
+          <t>RC0805FR-0710KL</t>
         </is>
       </c>
       <c r="I52" s="15" t="inlineStr">
         <is>
-          <t>81-BLM21PG601SN1D</t>
+          <t>603-RC0805FR-0710KL</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="15" t="inlineStr">
         <is>
-          <t>U7</t>
+          <t>R30</t>
         </is>
       </c>
       <c r="B53" s="15" t="inlineStr">
         <is>
-          <t>W5500</t>
+          <t>10kΩ</t>
         </is>
       </c>
       <c r="C53" s="15" t="inlineStr">
@@ -7495,35 +7185,39 @@
       </c>
       <c r="E53" s="15" t="inlineStr">
         <is>
-          <t>W5500:W5500</t>
+          <t>Device:R</t>
         </is>
       </c>
       <c r="F53" s="15" t="inlineStr">
         <is>
-          <t>W5500:48LQFP_W5500_WIZ</t>
+          <t>Resistor_SMD:R_0805_2012Metric</t>
         </is>
       </c>
       <c r="G53" s="15" t="inlineStr">
         <is>
-          <t>WIZnet</t>
+          <t>YAGEO</t>
         </is>
       </c>
       <c r="H53" s="15" t="inlineStr">
         <is>
-          <t>W5500</t>
-        </is>
-      </c>
-      <c r="I53" s="15" t="inlineStr"/>
+          <t>RC0805FR-0710KL</t>
+        </is>
+      </c>
+      <c r="I53" s="15" t="inlineStr">
+        <is>
+          <t>603-RC0805FR-0710KL</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="15" t="inlineStr">
         <is>
-          <t>R35</t>
+          <t>R31</t>
         </is>
       </c>
       <c r="B54" s="15" t="inlineStr">
         <is>
-          <t>0Ω</t>
+          <t>10kΩ</t>
         </is>
       </c>
       <c r="C54" s="15" t="inlineStr">
@@ -7553,24 +7247,24 @@
       </c>
       <c r="H54" s="15" t="inlineStr">
         <is>
-          <t>RC0805JR-070RL</t>
+          <t>RC0805FR-0710KL</t>
         </is>
       </c>
       <c r="I54" s="15" t="inlineStr">
         <is>
-          <t>603-RC0805JR-070RL</t>
+          <t>603-RC0805FR-0710KL</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="15" t="inlineStr">
         <is>
-          <t>R39</t>
+          <t>C24</t>
         </is>
       </c>
       <c r="B55" s="15" t="inlineStr">
         <is>
-          <t>49,9Ω 1%</t>
+          <t>10nF</t>
         </is>
       </c>
       <c r="C55" s="15" t="inlineStr">
@@ -7585,12 +7279,12 @@
       </c>
       <c r="E55" s="15" t="inlineStr">
         <is>
-          <t>Device:R</t>
+          <t>Device:C</t>
         </is>
       </c>
       <c r="F55" s="15" t="inlineStr">
         <is>
-          <t>Resistor_SMD:R_0805_2012Metric</t>
+          <t>Capacitor_SMD:C_0805_2012Metric</t>
         </is>
       </c>
       <c r="G55" s="15" t="inlineStr">
@@ -7600,29 +7294,29 @@
       </c>
       <c r="H55" s="15" t="inlineStr">
         <is>
-          <t>RC0805FR-0749R9L</t>
+          <t>CC0805KRX7R9BB103</t>
         </is>
       </c>
       <c r="I55" s="15" t="inlineStr">
         <is>
-          <t>603-RC0805FR-0749R9L</t>
+          <t>603-CC805KRX7R9BB103</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="15" t="inlineStr">
         <is>
-          <t>Y1</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="B56" s="15" t="inlineStr">
         <is>
-          <t>25 MHz</t>
+          <t>7499011121A</t>
         </is>
       </c>
       <c r="C56" s="15" t="inlineStr">
         <is>
-          <t>SMD</t>
+          <t>THT</t>
         </is>
       </c>
       <c r="D56" s="15" t="inlineStr">
@@ -7632,12 +7326,12 @@
       </c>
       <c r="E56" s="15" t="inlineStr">
         <is>
-          <t>wuerth_xtal:CFPX-104_830059532</t>
+          <t>wuerth_rj45:7499011121A</t>
         </is>
       </c>
       <c r="F56" s="15" t="inlineStr">
         <is>
-          <t>wuerth_830059532:Y_Wurth_WE-XTAL_Quartz-CFPX-104</t>
+          <t>wuerth_rj45:T_Wurth_WE-RJ45LAN_7499011121A</t>
         </is>
       </c>
       <c r="G56" s="15" t="inlineStr">
@@ -7647,24 +7341,24 @@
       </c>
       <c r="H56" s="15" t="inlineStr">
         <is>
-          <t>830059532</t>
+          <t>7499011121A</t>
         </is>
       </c>
       <c r="I56" s="15" t="inlineStr">
         <is>
-          <t>710-830059532</t>
+          <t>710-7499011121A</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="15" t="inlineStr">
         <is>
-          <t>C20</t>
+          <t>C23</t>
         </is>
       </c>
       <c r="B57" s="15" t="inlineStr">
         <is>
-          <t>100nF</t>
+          <t>4,7 µF</t>
         </is>
       </c>
       <c r="C57" s="15" t="inlineStr">
@@ -7689,29 +7383,29 @@
       </c>
       <c r="G57" s="15" t="inlineStr">
         <is>
-          <t>YAGEO</t>
+          <t>Samsung</t>
         </is>
       </c>
       <c r="H57" s="15" t="inlineStr">
         <is>
-          <t>CC0805KRX7R9BB104</t>
+          <t>CL21A475KAQNNNE</t>
         </is>
       </c>
       <c r="I57" s="15" t="inlineStr">
         <is>
-          <t>603-CC805KRX7R9BB104</t>
+          <t>187-CL21A475KAQNNNE</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="15" t="inlineStr">
         <is>
-          <t>R40</t>
+          <t>C31</t>
         </is>
       </c>
       <c r="B58" s="15" t="inlineStr">
         <is>
-          <t>49,9Ω 1%</t>
+          <t>10nF</t>
         </is>
       </c>
       <c r="C58" s="15" t="inlineStr">
@@ -7726,12 +7420,12 @@
       </c>
       <c r="E58" s="15" t="inlineStr">
         <is>
-          <t>Device:R</t>
+          <t>Device:C</t>
         </is>
       </c>
       <c r="F58" s="15" t="inlineStr">
         <is>
-          <t>Resistor_SMD:R_0805_2012Metric</t>
+          <t>Capacitor_SMD:C_0805_2012Metric</t>
         </is>
       </c>
       <c r="G58" s="15" t="inlineStr">
@@ -7741,24 +7435,24 @@
       </c>
       <c r="H58" s="15" t="inlineStr">
         <is>
-          <t>RC0805FR-0749R9L</t>
+          <t>CC0805KRX7R9BB103</t>
         </is>
       </c>
       <c r="I58" s="15" t="inlineStr">
         <is>
-          <t>603-RC0805FR-0749R9L</t>
+          <t>603-CC805KRX7R9BB103</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="15" t="inlineStr">
         <is>
-          <t>R27</t>
+          <t>C22</t>
         </is>
       </c>
       <c r="B59" s="15" t="inlineStr">
         <is>
-          <t>12,4kΩ, 1%</t>
+          <t>100nF</t>
         </is>
       </c>
       <c r="C59" s="15" t="inlineStr">
@@ -7773,12 +7467,12 @@
       </c>
       <c r="E59" s="15" t="inlineStr">
         <is>
-          <t>Device:R</t>
+          <t>Device:C</t>
         </is>
       </c>
       <c r="F59" s="15" t="inlineStr">
         <is>
-          <t>Resistor_SMD:R_0805_2012Metric</t>
+          <t>Capacitor_SMD:C_0805_2012Metric</t>
         </is>
       </c>
       <c r="G59" s="15" t="inlineStr">
@@ -7788,24 +7482,24 @@
       </c>
       <c r="H59" s="15" t="inlineStr">
         <is>
-          <t>RC0805FR-0712K4L</t>
+          <t>CC0805KRX7R9BB104</t>
         </is>
       </c>
       <c r="I59" s="15" t="inlineStr">
         <is>
-          <t>603-RC0805FR-0712K4L</t>
+          <t>603-CC805KRX7R9BB104</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="15" t="inlineStr">
         <is>
-          <t>R32</t>
+          <t>C30</t>
         </is>
       </c>
       <c r="B60" s="15" t="inlineStr">
         <is>
-          <t>10kΩ</t>
+          <t>6,8nF</t>
         </is>
       </c>
       <c r="C60" s="15" t="inlineStr">
@@ -7820,12 +7514,12 @@
       </c>
       <c r="E60" s="15" t="inlineStr">
         <is>
-          <t>Device:R</t>
+          <t>Device:C</t>
         </is>
       </c>
       <c r="F60" s="15" t="inlineStr">
         <is>
-          <t>Resistor_SMD:R_0805_2012Metric</t>
+          <t>Capacitor_SMD:C_0805_2012Metric</t>
         </is>
       </c>
       <c r="G60" s="15" t="inlineStr">
@@ -7835,24 +7529,24 @@
       </c>
       <c r="H60" s="15" t="inlineStr">
         <is>
-          <t>RC0805FR-0710KL</t>
+          <t>CC0805KRX7R9BB682</t>
         </is>
       </c>
       <c r="I60" s="15" t="inlineStr">
         <is>
-          <t>603-RC0805FR-0710KL</t>
+          <t>603-CC805KRX7R9BB682</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="15" t="inlineStr">
         <is>
-          <t>R30</t>
+          <t>C25</t>
         </is>
       </c>
       <c r="B61" s="15" t="inlineStr">
         <is>
-          <t>10kΩ</t>
+          <t>27 pF</t>
         </is>
       </c>
       <c r="C61" s="15" t="inlineStr">
@@ -7867,12 +7561,12 @@
       </c>
       <c r="E61" s="15" t="inlineStr">
         <is>
-          <t>Device:R</t>
+          <t>Device:C</t>
         </is>
       </c>
       <c r="F61" s="15" t="inlineStr">
         <is>
-          <t>Resistor_SMD:R_0805_2012Metric</t>
+          <t>Capacitor_SMD:C_0805_2012Metric</t>
         </is>
       </c>
       <c r="G61" s="15" t="inlineStr">
@@ -7882,19 +7576,19 @@
       </c>
       <c r="H61" s="15" t="inlineStr">
         <is>
-          <t>RC0805FR-0710KL</t>
+          <t>CC0805JRNPO9BN270</t>
         </is>
       </c>
       <c r="I61" s="15" t="inlineStr">
         <is>
-          <t>603-RC0805FR-0710KL</t>
+          <t>603-CC805JRNPO9BN270</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="15" t="inlineStr">
         <is>
-          <t>R31</t>
+          <t>R28</t>
         </is>
       </c>
       <c r="B62" s="15" t="inlineStr">
@@ -7941,12 +7635,12 @@
     <row r="63">
       <c r="A63" s="15" t="inlineStr">
         <is>
-          <t>C24</t>
+          <t>R36</t>
         </is>
       </c>
       <c r="B63" s="15" t="inlineStr">
         <is>
-          <t>10nF</t>
+          <t>49,9Ω 1%</t>
         </is>
       </c>
       <c r="C63" s="15" t="inlineStr">
@@ -7961,12 +7655,12 @@
       </c>
       <c r="E63" s="15" t="inlineStr">
         <is>
-          <t>Device:C</t>
+          <t>Device:R</t>
         </is>
       </c>
       <c r="F63" s="15" t="inlineStr">
         <is>
-          <t>Capacitor_SMD:C_0805_2012Metric</t>
+          <t>Resistor_SMD:R_0805_2012Metric</t>
         </is>
       </c>
       <c r="G63" s="15" t="inlineStr">
@@ -7976,29 +7670,29 @@
       </c>
       <c r="H63" s="15" t="inlineStr">
         <is>
-          <t>CC0805KRX7R9BB103</t>
+          <t>RC0805FR-0749R9L</t>
         </is>
       </c>
       <c r="I63" s="15" t="inlineStr">
         <is>
-          <t>603-CC805KRX7R9BB103</t>
+          <t>603-RC0805FR-0749R9L</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="15" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>R37</t>
         </is>
       </c>
       <c r="B64" s="15" t="inlineStr">
         <is>
-          <t>7499011121A</t>
+          <t>49,9Ω 1%</t>
         </is>
       </c>
       <c r="C64" s="15" t="inlineStr">
         <is>
-          <t>THT</t>
+          <t>SMD</t>
         </is>
       </c>
       <c r="D64" s="15" t="inlineStr">
@@ -8008,39 +7702,39 @@
       </c>
       <c r="E64" s="15" t="inlineStr">
         <is>
-          <t>wuerth_rj45:7499011121A</t>
+          <t>Device:R</t>
         </is>
       </c>
       <c r="F64" s="15" t="inlineStr">
         <is>
-          <t>wuerth_rj45:T_Wurth_WE-RJ45LAN_7499011121A</t>
+          <t>Resistor_SMD:R_0805_2012Metric</t>
         </is>
       </c>
       <c r="G64" s="15" t="inlineStr">
         <is>
-          <t>Wurth Elektronik</t>
+          <t>YAGEO</t>
         </is>
       </c>
       <c r="H64" s="15" t="inlineStr">
         <is>
-          <t>7499011121A</t>
+          <t>RC0805FR-0749R9L</t>
         </is>
       </c>
       <c r="I64" s="15" t="inlineStr">
         <is>
-          <t>710-7499011121A</t>
+          <t>603-RC0805FR-0749R9L</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="15" t="inlineStr">
         <is>
-          <t>C23</t>
+          <t>R38</t>
         </is>
       </c>
       <c r="B65" s="15" t="inlineStr">
         <is>
-          <t>4,7 µF</t>
+          <t>10Ω 1%</t>
         </is>
       </c>
       <c r="C65" s="15" t="inlineStr">
@@ -8055,39 +7749,39 @@
       </c>
       <c r="E65" s="15" t="inlineStr">
         <is>
-          <t>Device:C</t>
+          <t>Device:R</t>
         </is>
       </c>
       <c r="F65" s="15" t="inlineStr">
         <is>
-          <t>Capacitor_SMD:C_0805_2012Metric</t>
+          <t>Resistor_SMD:R_0805_2012Metric</t>
         </is>
       </c>
       <c r="G65" s="15" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>YAGEO</t>
         </is>
       </c>
       <c r="H65" s="15" t="inlineStr">
         <is>
-          <t>CL21A475KAQNNNE</t>
+          <t>RC0805FR-0710RL</t>
         </is>
       </c>
       <c r="I65" s="15" t="inlineStr">
         <is>
-          <t>187-CL21A475KAQNNNE</t>
+          <t>603-RC0805FR-0710RL</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="15" t="inlineStr">
         <is>
-          <t>C31</t>
+          <t>R29</t>
         </is>
       </c>
       <c r="B66" s="15" t="inlineStr">
         <is>
-          <t>10nF</t>
+          <t>10kΩ</t>
         </is>
       </c>
       <c r="C66" s="15" t="inlineStr">
@@ -8102,12 +7796,12 @@
       </c>
       <c r="E66" s="15" t="inlineStr">
         <is>
-          <t>Device:C</t>
+          <t>Device:R</t>
         </is>
       </c>
       <c r="F66" s="15" t="inlineStr">
         <is>
-          <t>Capacitor_SMD:C_0805_2012Metric</t>
+          <t>Resistor_SMD:R_0805_2012Metric</t>
         </is>
       </c>
       <c r="G66" s="15" t="inlineStr">
@@ -8117,24 +7811,24 @@
       </c>
       <c r="H66" s="15" t="inlineStr">
         <is>
-          <t>CC0805KRX7R9BB103</t>
+          <t>RC0805FR-0710KL</t>
         </is>
       </c>
       <c r="I66" s="15" t="inlineStr">
         <is>
-          <t>603-CC805KRX7R9BB103</t>
+          <t>603-RC0805FR-0710KL</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="15" t="inlineStr">
         <is>
-          <t>C22</t>
+          <t>C32</t>
         </is>
       </c>
       <c r="B67" s="15" t="inlineStr">
         <is>
-          <t>100nF</t>
+          <t>22nF</t>
         </is>
       </c>
       <c r="C67" s="15" t="inlineStr">
@@ -8159,29 +7853,29 @@
       </c>
       <c r="G67" s="15" t="inlineStr">
         <is>
-          <t>YAGEO</t>
+          <t>Samsung</t>
         </is>
       </c>
       <c r="H67" s="15" t="inlineStr">
         <is>
-          <t>CC0805KRX7R9BB104</t>
+          <t>CL21B223KBANNNC</t>
         </is>
       </c>
       <c r="I67" s="15" t="inlineStr">
         <is>
-          <t>603-CC805KRX7R9BB104</t>
+          <t>187-CL21B223KBANNNC</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="15" t="inlineStr">
         <is>
-          <t>C30</t>
+          <t>C26</t>
         </is>
       </c>
       <c r="B68" s="15" t="inlineStr">
         <is>
-          <t>6,8nF</t>
+          <t>27 pF</t>
         </is>
       </c>
       <c r="C68" s="15" t="inlineStr">
@@ -8211,24 +7905,24 @@
       </c>
       <c r="H68" s="15" t="inlineStr">
         <is>
-          <t>CC0805KRX7R9BB682</t>
+          <t>CC0805JRNPO9BN270</t>
         </is>
       </c>
       <c r="I68" s="15" t="inlineStr">
         <is>
-          <t>603-CC805KRX7R9BB682</t>
+          <t>603-CC805JRNPO9BN270</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="15" t="inlineStr">
         <is>
-          <t>C25</t>
+          <t>C29</t>
         </is>
       </c>
       <c r="B69" s="15" t="inlineStr">
         <is>
-          <t>27 pF</t>
+          <t>6,8nF</t>
         </is>
       </c>
       <c r="C69" s="15" t="inlineStr">
@@ -8258,24 +7952,24 @@
       </c>
       <c r="H69" s="15" t="inlineStr">
         <is>
-          <t>CC0805JRNPO9BN270</t>
+          <t>CC0805KRX7R9BB682</t>
         </is>
       </c>
       <c r="I69" s="15" t="inlineStr">
         <is>
-          <t>603-CC805JRNPO9BN270</t>
+          <t>603-CC805KRX7R9BB682</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="15" t="inlineStr">
         <is>
-          <t>R28</t>
+          <t>C19</t>
         </is>
       </c>
       <c r="B70" s="15" t="inlineStr">
         <is>
-          <t>10kΩ</t>
+          <t>100nF</t>
         </is>
       </c>
       <c r="C70" s="15" t="inlineStr">
@@ -8290,12 +7984,12 @@
       </c>
       <c r="E70" s="15" t="inlineStr">
         <is>
-          <t>Device:R</t>
+          <t>Device:C</t>
         </is>
       </c>
       <c r="F70" s="15" t="inlineStr">
         <is>
-          <t>Resistor_SMD:R_0805_2012Metric</t>
+          <t>Capacitor_SMD:C_0805_2012Metric</t>
         </is>
       </c>
       <c r="G70" s="15" t="inlineStr">
@@ -8305,24 +7999,24 @@
       </c>
       <c r="H70" s="15" t="inlineStr">
         <is>
-          <t>RC0805FR-0710KL</t>
+          <t>CC0805KRX7R9BB104</t>
         </is>
       </c>
       <c r="I70" s="15" t="inlineStr">
         <is>
-          <t>603-RC0805FR-0710KL</t>
+          <t>603-CC805KRX7R9BB104</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="15" t="inlineStr">
         <is>
-          <t>R36</t>
+          <t>C27</t>
         </is>
       </c>
       <c r="B71" s="15" t="inlineStr">
         <is>
-          <t>49,9Ω 1%</t>
+          <t>10 µF</t>
         </is>
       </c>
       <c r="C71" s="15" t="inlineStr">
@@ -8337,39 +8031,39 @@
       </c>
       <c r="E71" s="15" t="inlineStr">
         <is>
-          <t>Device:R</t>
+          <t>Device:C</t>
         </is>
       </c>
       <c r="F71" s="15" t="inlineStr">
         <is>
-          <t>Resistor_SMD:R_0805_2012Metric</t>
+          <t>Capacitor_SMD:C_0805_2012Metric</t>
         </is>
       </c>
       <c r="G71" s="15" t="inlineStr">
         <is>
-          <t>YAGEO</t>
+          <t>Samsung</t>
         </is>
       </c>
       <c r="H71" s="15" t="inlineStr">
         <is>
-          <t>RC0805FR-0749R9L</t>
+          <t>CL21B106KOQNNNE</t>
         </is>
       </c>
       <c r="I71" s="15" t="inlineStr">
         <is>
-          <t>603-RC0805FR-0749R9L</t>
+          <t>187-CL21B106KOQNNNE</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="15" t="inlineStr">
         <is>
-          <t>R37</t>
+          <t>C18</t>
         </is>
       </c>
       <c r="B72" s="15" t="inlineStr">
         <is>
-          <t>49,9Ω 1%</t>
+          <t>100nF</t>
         </is>
       </c>
       <c r="C72" s="15" t="inlineStr">
@@ -8384,12 +8078,12 @@
       </c>
       <c r="E72" s="15" t="inlineStr">
         <is>
-          <t>Device:R</t>
+          <t>Device:C</t>
         </is>
       </c>
       <c r="F72" s="15" t="inlineStr">
         <is>
-          <t>Resistor_SMD:R_0805_2012Metric</t>
+          <t>Capacitor_SMD:C_0805_2012Metric</t>
         </is>
       </c>
       <c r="G72" s="15" t="inlineStr">
@@ -8399,24 +8093,24 @@
       </c>
       <c r="H72" s="15" t="inlineStr">
         <is>
-          <t>RC0805FR-0749R9L</t>
+          <t>CC0805KRX7R9BB104</t>
         </is>
       </c>
       <c r="I72" s="15" t="inlineStr">
         <is>
-          <t>603-RC0805FR-0749R9L</t>
+          <t>603-CC805KRX7R9BB104</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="15" t="inlineStr">
         <is>
-          <t>R38</t>
+          <t>C21</t>
         </is>
       </c>
       <c r="B73" s="15" t="inlineStr">
         <is>
-          <t>10Ω 1%</t>
+          <t>100nF</t>
         </is>
       </c>
       <c r="C73" s="15" t="inlineStr">
@@ -8431,12 +8125,12 @@
       </c>
       <c r="E73" s="15" t="inlineStr">
         <is>
-          <t>Device:R</t>
+          <t>Device:C</t>
         </is>
       </c>
       <c r="F73" s="15" t="inlineStr">
         <is>
-          <t>Resistor_SMD:R_0805_2012Metric</t>
+          <t>Capacitor_SMD:C_0805_2012Metric</t>
         </is>
       </c>
       <c r="G73" s="15" t="inlineStr">
@@ -8446,24 +8140,24 @@
       </c>
       <c r="H73" s="15" t="inlineStr">
         <is>
-          <t>RC0805FR-0710RL</t>
+          <t>CC0805KRX7R9BB104</t>
         </is>
       </c>
       <c r="I73" s="15" t="inlineStr">
         <is>
-          <t>603-RC0805FR-0710RL</t>
+          <t>603-CC805KRX7R9BB104</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="15" t="inlineStr">
         <is>
-          <t>R29</t>
+          <t>C17</t>
         </is>
       </c>
       <c r="B74" s="15" t="inlineStr">
         <is>
-          <t>10kΩ</t>
+          <t>100nF</t>
         </is>
       </c>
       <c r="C74" s="15" t="inlineStr">
@@ -8478,12 +8172,12 @@
       </c>
       <c r="E74" s="15" t="inlineStr">
         <is>
-          <t>Device:R</t>
+          <t>Device:C</t>
         </is>
       </c>
       <c r="F74" s="15" t="inlineStr">
         <is>
-          <t>Resistor_SMD:R_0805_2012Metric</t>
+          <t>Capacitor_SMD:C_0805_2012Metric</t>
         </is>
       </c>
       <c r="G74" s="15" t="inlineStr">
@@ -8493,24 +8187,24 @@
       </c>
       <c r="H74" s="15" t="inlineStr">
         <is>
-          <t>RC0805FR-0710KL</t>
+          <t>CC0805KRX7R9BB104</t>
         </is>
       </c>
       <c r="I74" s="15" t="inlineStr">
         <is>
-          <t>603-RC0805FR-0710KL</t>
+          <t>603-CC805KRX7R9BB104</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="15" t="inlineStr">
         <is>
-          <t>C32</t>
+          <t>C28</t>
         </is>
       </c>
       <c r="B75" s="15" t="inlineStr">
         <is>
-          <t>22nF</t>
+          <t>1nF/2kV</t>
         </is>
       </c>
       <c r="C75" s="15" t="inlineStr">
@@ -8530,403 +8224,27 @@
       </c>
       <c r="F75" s="15" t="inlineStr">
         <is>
-          <t>Capacitor_SMD:C_0805_2012Metric</t>
+          <t>Capacitor_SMD:C_1206_3216Metric</t>
         </is>
       </c>
       <c r="G75" s="15" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>KEMET</t>
         </is>
       </c>
       <c r="H75" s="15" t="inlineStr">
         <is>
-          <t>CL21B223KBANNNC</t>
+          <t>C1206C102KGRACTU</t>
         </is>
       </c>
       <c r="I75" s="15" t="inlineStr">
         <is>
-          <t>187-CL21B223KBANNNC</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" s="15" t="inlineStr">
-        <is>
-          <t>C26</t>
-        </is>
-      </c>
-      <c r="B76" s="15" t="inlineStr">
-        <is>
-          <t>27 pF</t>
-        </is>
-      </c>
-      <c r="C76" s="15" t="inlineStr">
-        <is>
-          <t>SMD</t>
-        </is>
-      </c>
-      <c r="D76" s="15" t="inlineStr">
-        <is>
-          <t>ethernet.kicad_sch</t>
-        </is>
-      </c>
-      <c r="E76" s="15" t="inlineStr">
-        <is>
-          <t>Device:C</t>
-        </is>
-      </c>
-      <c r="F76" s="15" t="inlineStr">
-        <is>
-          <t>Capacitor_SMD:C_0805_2012Metric</t>
-        </is>
-      </c>
-      <c r="G76" s="15" t="inlineStr">
-        <is>
-          <t>YAGEO</t>
-        </is>
-      </c>
-      <c r="H76" s="15" t="inlineStr">
-        <is>
-          <t>CC0805JRNPO9BN270</t>
-        </is>
-      </c>
-      <c r="I76" s="15" t="inlineStr">
-        <is>
-          <t>603-CC805JRNPO9BN270</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" s="15" t="inlineStr">
-        <is>
-          <t>C29</t>
-        </is>
-      </c>
-      <c r="B77" s="15" t="inlineStr">
-        <is>
-          <t>6,8nF</t>
-        </is>
-      </c>
-      <c r="C77" s="15" t="inlineStr">
-        <is>
-          <t>SMD</t>
-        </is>
-      </c>
-      <c r="D77" s="15" t="inlineStr">
-        <is>
-          <t>ethernet.kicad_sch</t>
-        </is>
-      </c>
-      <c r="E77" s="15" t="inlineStr">
-        <is>
-          <t>Device:C</t>
-        </is>
-      </c>
-      <c r="F77" s="15" t="inlineStr">
-        <is>
-          <t>Capacitor_SMD:C_0805_2012Metric</t>
-        </is>
-      </c>
-      <c r="G77" s="15" t="inlineStr">
-        <is>
-          <t>YAGEO</t>
-        </is>
-      </c>
-      <c r="H77" s="15" t="inlineStr">
-        <is>
-          <t>CC0805KRX7R9BB682</t>
-        </is>
-      </c>
-      <c r="I77" s="15" t="inlineStr">
-        <is>
-          <t>603-CC805KRX7R9BB682</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" s="15" t="inlineStr">
-        <is>
-          <t>C19</t>
-        </is>
-      </c>
-      <c r="B78" s="15" t="inlineStr">
-        <is>
-          <t>100nF</t>
-        </is>
-      </c>
-      <c r="C78" s="15" t="inlineStr">
-        <is>
-          <t>SMD</t>
-        </is>
-      </c>
-      <c r="D78" s="15" t="inlineStr">
-        <is>
-          <t>ethernet.kicad_sch</t>
-        </is>
-      </c>
-      <c r="E78" s="15" t="inlineStr">
-        <is>
-          <t>Device:C</t>
-        </is>
-      </c>
-      <c r="F78" s="15" t="inlineStr">
-        <is>
-          <t>Capacitor_SMD:C_0805_2012Metric</t>
-        </is>
-      </c>
-      <c r="G78" s="15" t="inlineStr">
-        <is>
-          <t>YAGEO</t>
-        </is>
-      </c>
-      <c r="H78" s="15" t="inlineStr">
-        <is>
-          <t>CC0805KRX7R9BB104</t>
-        </is>
-      </c>
-      <c r="I78" s="15" t="inlineStr">
-        <is>
-          <t>603-CC805KRX7R9BB104</t>
-        </is>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" s="15" t="inlineStr">
-        <is>
-          <t>C27</t>
-        </is>
-      </c>
-      <c r="B79" s="15" t="inlineStr">
-        <is>
-          <t>10 µF</t>
-        </is>
-      </c>
-      <c r="C79" s="15" t="inlineStr">
-        <is>
-          <t>SMD</t>
-        </is>
-      </c>
-      <c r="D79" s="15" t="inlineStr">
-        <is>
-          <t>ethernet.kicad_sch</t>
-        </is>
-      </c>
-      <c r="E79" s="15" t="inlineStr">
-        <is>
-          <t>Device:C</t>
-        </is>
-      </c>
-      <c r="F79" s="15" t="inlineStr">
-        <is>
-          <t>Capacitor_SMD:C_0805_2012Metric</t>
-        </is>
-      </c>
-      <c r="G79" s="15" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="H79" s="15" t="inlineStr">
-        <is>
-          <t>CL21B106KOQNNNE</t>
-        </is>
-      </c>
-      <c r="I79" s="15" t="inlineStr">
-        <is>
-          <t>187-CL21B106KOQNNNE</t>
-        </is>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" s="15" t="inlineStr">
-        <is>
-          <t>C18</t>
-        </is>
-      </c>
-      <c r="B80" s="15" t="inlineStr">
-        <is>
-          <t>100nF</t>
-        </is>
-      </c>
-      <c r="C80" s="15" t="inlineStr">
-        <is>
-          <t>SMD</t>
-        </is>
-      </c>
-      <c r="D80" s="15" t="inlineStr">
-        <is>
-          <t>ethernet.kicad_sch</t>
-        </is>
-      </c>
-      <c r="E80" s="15" t="inlineStr">
-        <is>
-          <t>Device:C</t>
-        </is>
-      </c>
-      <c r="F80" s="15" t="inlineStr">
-        <is>
-          <t>Capacitor_SMD:C_0805_2012Metric</t>
-        </is>
-      </c>
-      <c r="G80" s="15" t="inlineStr">
-        <is>
-          <t>YAGEO</t>
-        </is>
-      </c>
-      <c r="H80" s="15" t="inlineStr">
-        <is>
-          <t>CC0805KRX7R9BB104</t>
-        </is>
-      </c>
-      <c r="I80" s="15" t="inlineStr">
-        <is>
-          <t>603-CC805KRX7R9BB104</t>
-        </is>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" s="15" t="inlineStr">
-        <is>
-          <t>C21</t>
-        </is>
-      </c>
-      <c r="B81" s="15" t="inlineStr">
-        <is>
-          <t>100nF</t>
-        </is>
-      </c>
-      <c r="C81" s="15" t="inlineStr">
-        <is>
-          <t>SMD</t>
-        </is>
-      </c>
-      <c r="D81" s="15" t="inlineStr">
-        <is>
-          <t>ethernet.kicad_sch</t>
-        </is>
-      </c>
-      <c r="E81" s="15" t="inlineStr">
-        <is>
-          <t>Device:C</t>
-        </is>
-      </c>
-      <c r="F81" s="15" t="inlineStr">
-        <is>
-          <t>Capacitor_SMD:C_0805_2012Metric</t>
-        </is>
-      </c>
-      <c r="G81" s="15" t="inlineStr">
-        <is>
-          <t>YAGEO</t>
-        </is>
-      </c>
-      <c r="H81" s="15" t="inlineStr">
-        <is>
-          <t>CC0805KRX7R9BB104</t>
-        </is>
-      </c>
-      <c r="I81" s="15" t="inlineStr">
-        <is>
-          <t>603-CC805KRX7R9BB104</t>
-        </is>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" s="15" t="inlineStr">
-        <is>
-          <t>C17</t>
-        </is>
-      </c>
-      <c r="B82" s="15" t="inlineStr">
-        <is>
-          <t>100nF</t>
-        </is>
-      </c>
-      <c r="C82" s="15" t="inlineStr">
-        <is>
-          <t>SMD</t>
-        </is>
-      </c>
-      <c r="D82" s="15" t="inlineStr">
-        <is>
-          <t>ethernet.kicad_sch</t>
-        </is>
-      </c>
-      <c r="E82" s="15" t="inlineStr">
-        <is>
-          <t>Device:C</t>
-        </is>
-      </c>
-      <c r="F82" s="15" t="inlineStr">
-        <is>
-          <t>Capacitor_SMD:C_0805_2012Metric</t>
-        </is>
-      </c>
-      <c r="G82" s="15" t="inlineStr">
-        <is>
-          <t>YAGEO</t>
-        </is>
-      </c>
-      <c r="H82" s="15" t="inlineStr">
-        <is>
-          <t>CC0805KRX7R9BB104</t>
-        </is>
-      </c>
-      <c r="I82" s="15" t="inlineStr">
-        <is>
-          <t>603-CC805KRX7R9BB104</t>
-        </is>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" s="15" t="inlineStr">
-        <is>
-          <t>C28</t>
-        </is>
-      </c>
-      <c r="B83" s="15" t="inlineStr">
-        <is>
-          <t>1nF/2kV</t>
-        </is>
-      </c>
-      <c r="C83" s="15" t="inlineStr">
-        <is>
-          <t>SMD</t>
-        </is>
-      </c>
-      <c r="D83" s="15" t="inlineStr">
-        <is>
-          <t>ethernet.kicad_sch</t>
-        </is>
-      </c>
-      <c r="E83" s="15" t="inlineStr">
-        <is>
-          <t>Device:C</t>
-        </is>
-      </c>
-      <c r="F83" s="15" t="inlineStr">
-        <is>
-          <t>Capacitor_SMD:C_1206_3216Metric</t>
-        </is>
-      </c>
-      <c r="G83" s="15" t="inlineStr">
-        <is>
-          <t>KEMET</t>
-        </is>
-      </c>
-      <c r="H83" s="15" t="inlineStr">
-        <is>
-          <t>C1206C102KGRACTU</t>
-        </is>
-      </c>
-      <c r="I83" s="15" t="inlineStr">
-        <is>
           <t>80-C1206C102KGR</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A5:I83"/>
+  <autoFilter ref="A5:I75"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -8957,7 +8275,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Stand 2026-09-29 · Der Schaltplan ist elektrisch fertig (ERC 0 Fehler).</t>
+          <t>Stand 2026-09-30 · Der Schaltplan ist elektrisch fertig (ERC 0 Fehler).</t>
         </is>
       </c>
     </row>
@@ -9051,17 +8369,17 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Mischbestückung THT / SMD (22 bedrahtete Teile)</t>
+          <t>Mischbestückung THT / SMD (5 bedrahtete Teile)</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Bedrahtet: D7, D8, D9, D10, J1, J6, J_PWR1, Q1, Q2, Q3, Q4, R9, R13, R14, R15, R16, R23, R24, R25, R26, S2, T1.</t>
+          <t>Bedrahtet: J1, J6, J_PWR1, S2, T1.</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Bedrahtete Teile erzwingen einen zweiten Bestückungsdurchlauf und verteuern die Fertigung spürbar. R13–R16 und R23–R26 sitzen zudem im Footprint DIN0617 (17 mm, 2-W-Klasse) — für 220 Ω und 4,7 kΩ in einer Signalfunktion überdimensioniert. Bei den LEDs und Steckverbindern ist THT bewusst gewählt; zu prüfen ist vor allem, ob Q1–Q4 und die Widerstände SMD werden können.</t>
+          <t>Bedrahtete Teile erzwingen einen zweiten Bestückungsdurchlauf und verteuern die Fertigung spürbar. Die LED-Treiberstufe (Q1–Q4, R23–R26) ist seit SHBS-40 entfallen, R9 und R13–R16 sind 0805. Bei den LEDs, Elkos und Steckverbindern ist THT bewusst gewählt.</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">

</xml_diff>